<commit_message>
Add missing Foodex2 codes to codes file
I used the EFSA Catalogue Browser 1.2.19 and the MTX catalogue (17.2).
</commit_message>
<xml_diff>
--- a/data-preprocessing/codes/rpc-to-sua.xlsx
+++ b/data-preprocessing/codes/rpc-to-sua.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wilhelmwanecek/dev/safad/data-preprocessing/codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9381EC20-42BE-5E49-9FF0-6AE591EA53BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E380338E-4A65-5F49-8568-56906519F3A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="26540" windowHeight="16700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2724" uniqueCount="1556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2746" uniqueCount="1577">
   <si>
     <t>FoodEx2 Code</t>
   </si>
@@ -4708,6 +4708,69 @@
   </si>
   <si>
     <t>Comment</t>
+  </si>
+  <si>
+    <t>A01LC</t>
+  </si>
+  <si>
+    <t>A01DB</t>
+  </si>
+  <si>
+    <t>A01FV</t>
+  </si>
+  <si>
+    <t>A01FL</t>
+  </si>
+  <si>
+    <t>A01EJ</t>
+  </si>
+  <si>
+    <t>A01LR</t>
+  </si>
+  <si>
+    <t>A001JZ</t>
+  </si>
+  <si>
+    <t>A016P</t>
+  </si>
+  <si>
+    <t>A016N</t>
+  </si>
+  <si>
+    <t>A018F</t>
+  </si>
+  <si>
+    <t>A00VY</t>
+  </si>
+  <si>
+    <t>A05SG</t>
+  </si>
+  <si>
+    <t>A0BB7</t>
+  </si>
+  <si>
+    <t>A034A</t>
+  </si>
+  <si>
+    <t>A16XV</t>
+  </si>
+  <si>
+    <t>A0ESB</t>
+  </si>
+  <si>
+    <t>A06CE</t>
+  </si>
+  <si>
+    <t>A0488B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could not find exact fx2 match, chose "Acid" (in fod dditives) </t>
+  </si>
+  <si>
+    <t>A03SR</t>
+  </si>
+  <si>
+    <t>A033H</t>
   </si>
 </sst>
 </file>
@@ -4936,7 +4999,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -5036,27 +5099,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="14">
     <cellStyle name="Hyperlink" xfId="11" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -5074,297 +5134,7 @@
     <cellStyle name="Normal 7" xfId="8" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
     <cellStyle name="Validate" xfId="5" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
   </cellStyles>
-  <dxfs count="35">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5740,7 +5510,7 @@
   <cols>
     <col min="1" max="2" width="18.5" style="17" customWidth="1"/>
     <col min="3" max="3" width="33.5" customWidth="1"/>
-    <col min="4" max="4" width="19" style="43" customWidth="1"/>
+    <col min="4" max="4" width="19" style="15" customWidth="1"/>
     <col min="5" max="5" width="46.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5754,7 +5524,7 @@
       <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="43" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="12" t="s">
@@ -5777,7 +5547,7 @@
       <c r="C2" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="D2" s="15" t="s">
         <v>201</v>
       </c>
       <c r="E2" t="s">
@@ -5797,7 +5567,7 @@
       <c r="C3" s="4" t="s">
         <v>399</v>
       </c>
-      <c r="D3" s="43" t="s">
+      <c r="D3" s="15" t="s">
         <v>201</v>
       </c>
       <c r="E3" t="s">
@@ -5817,7 +5587,7 @@
       <c r="C4" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="D4" s="43" t="s">
+      <c r="D4" s="15" t="s">
         <v>201</v>
       </c>
       <c r="E4" t="s">
@@ -5837,7 +5607,7 @@
       <c r="C5" s="4" t="s">
         <v>1275</v>
       </c>
-      <c r="D5" s="43" t="s">
+      <c r="D5" s="15" t="s">
         <v>201</v>
       </c>
       <c r="E5" t="s">
@@ -5857,7 +5627,7 @@
       <c r="C6" s="4" t="s">
         <v>1425</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="15" t="s">
         <v>201</v>
       </c>
       <c r="E6" t="s">
@@ -5877,7 +5647,7 @@
       <c r="C7" s="4" t="s">
         <v>826</v>
       </c>
-      <c r="D7" s="43" t="s">
+      <c r="D7" s="15" t="s">
         <v>827</v>
       </c>
       <c r="E7" t="s">
@@ -5897,7 +5667,7 @@
       <c r="C8" s="4" t="s">
         <v>697</v>
       </c>
-      <c r="D8" s="43" t="s">
+      <c r="D8" s="15" t="s">
         <v>698</v>
       </c>
       <c r="E8" t="s">
@@ -5917,7 +5687,7 @@
       <c r="C9" s="4" t="s">
         <v>1143</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="15" t="s">
         <v>698</v>
       </c>
       <c r="E9" t="s">
@@ -5937,7 +5707,7 @@
       <c r="C10" s="34" t="s">
         <v>1261</v>
       </c>
-      <c r="D10" s="44" t="s">
+      <c r="D10" s="43" t="s">
         <v>1262</v>
       </c>
       <c r="E10" s="34" t="s">
@@ -5955,7 +5725,7 @@
       <c r="C11" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D11" s="43" t="s">
+      <c r="D11" s="15" t="s">
         <v>106</v>
       </c>
       <c r="E11" t="s">
@@ -5975,7 +5745,7 @@
       <c r="C12" s="4" t="s">
         <v>1159</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="15" t="s">
         <v>1160</v>
       </c>
       <c r="E12" t="s">
@@ -5995,7 +5765,7 @@
       <c r="C13" s="4" t="s">
         <v>932</v>
       </c>
-      <c r="D13" s="43" t="s">
+      <c r="D13" s="15" t="s">
         <v>933</v>
       </c>
       <c r="E13" t="s">
@@ -6015,7 +5785,7 @@
       <c r="C14" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="15" t="s">
         <v>387</v>
       </c>
       <c r="E14" t="s">
@@ -6035,7 +5805,7 @@
       <c r="C15" s="34" t="s">
         <v>876</v>
       </c>
-      <c r="D15" s="43" t="s">
+      <c r="D15" s="15" t="s">
         <v>387</v>
       </c>
       <c r="E15" t="s">
@@ -6057,7 +5827,7 @@
       <c r="C16" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="D16" s="43" t="s">
+      <c r="D16" s="15" t="s">
         <v>196</v>
       </c>
       <c r="E16" t="s">
@@ -6077,7 +5847,7 @@
       <c r="C17" s="4" t="s">
         <v>1111</v>
       </c>
-      <c r="D17" s="43" t="s">
+      <c r="D17" s="15" t="s">
         <v>1112</v>
       </c>
       <c r="E17" s="2" t="s">
@@ -6097,7 +5867,7 @@
       <c r="C18" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="43" t="s">
+      <c r="D18" s="15" t="s">
         <v>68</v>
       </c>
       <c r="E18" t="s">
@@ -6117,7 +5887,7 @@
       <c r="C19" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="D19" s="43" t="s">
+      <c r="D19" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E19" t="s">
@@ -6137,7 +5907,7 @@
       <c r="C20" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="D20" s="43" t="s">
+      <c r="D20" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E20" t="s">
@@ -6157,7 +5927,7 @@
       <c r="C21" s="4" t="s">
         <v>427</v>
       </c>
-      <c r="D21" s="43" t="s">
+      <c r="D21" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E21" t="s">
@@ -6177,7 +5947,7 @@
       <c r="C22" s="4" t="s">
         <v>651</v>
       </c>
-      <c r="D22" s="43" t="s">
+      <c r="D22" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E22" t="s">
@@ -6197,7 +5967,7 @@
       <c r="C23" s="4" t="s">
         <v>714</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E23" t="s">
@@ -6217,7 +5987,7 @@
       <c r="C24" s="4" t="s">
         <v>722</v>
       </c>
-      <c r="D24" s="43" t="s">
+      <c r="D24" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E24" t="s">
@@ -6237,7 +6007,7 @@
       <c r="C25" s="4" t="s">
         <v>741</v>
       </c>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E25" t="s">
@@ -6257,7 +6027,7 @@
       <c r="C26" s="4" t="s">
         <v>1119</v>
       </c>
-      <c r="D26" s="43" t="s">
+      <c r="D26" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E26" t="s">
@@ -6277,7 +6047,7 @@
       <c r="C27" s="4" t="s">
         <v>1150</v>
       </c>
-      <c r="D27" s="43" t="s">
+      <c r="D27" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E27" t="s">
@@ -6297,7 +6067,7 @@
       <c r="C28" s="4" t="s">
         <v>1323</v>
       </c>
-      <c r="D28" s="43" t="s">
+      <c r="D28" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E28" t="s">
@@ -6317,7 +6087,7 @@
       <c r="C29" s="4" t="s">
         <v>1415</v>
       </c>
-      <c r="D29" s="43" t="s">
+      <c r="D29" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E29" t="s">
@@ -6337,7 +6107,7 @@
       <c r="C30" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="D30" s="43" t="s">
+      <c r="D30" s="15" t="s">
         <v>186</v>
       </c>
       <c r="E30" t="s">
@@ -6357,7 +6127,7 @@
       <c r="C31" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="D31" s="43" t="s">
+      <c r="D31" s="15" t="s">
         <v>186</v>
       </c>
       <c r="E31" t="s">
@@ -6377,7 +6147,7 @@
       <c r="C32" s="4" t="s">
         <v>430</v>
       </c>
-      <c r="D32" s="43" t="s">
+      <c r="D32" s="15" t="s">
         <v>431</v>
       </c>
       <c r="E32" t="s">
@@ -6397,7 +6167,7 @@
       <c r="C33" s="4" t="s">
         <v>505</v>
       </c>
-      <c r="D33" s="43" t="s">
+      <c r="D33" s="15" t="s">
         <v>431</v>
       </c>
       <c r="E33" t="s">
@@ -6417,7 +6187,7 @@
       <c r="C34" s="4" t="s">
         <v>654</v>
       </c>
-      <c r="D34" s="43" t="s">
+      <c r="D34" s="15" t="s">
         <v>431</v>
       </c>
       <c r="E34" t="s">
@@ -6437,7 +6207,7 @@
       <c r="C35" s="4" t="s">
         <v>738</v>
       </c>
-      <c r="D35" s="43" t="s">
+      <c r="D35" s="15" t="s">
         <v>431</v>
       </c>
       <c r="E35" t="s">
@@ -6457,7 +6227,7 @@
       <c r="C36" s="4" t="s">
         <v>1455</v>
       </c>
-      <c r="D36" s="43" t="s">
+      <c r="D36" s="15" t="s">
         <v>431</v>
       </c>
       <c r="E36" s="17" t="s">
@@ -6480,7 +6250,7 @@
       <c r="C37" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="D37" s="43" t="s">
+      <c r="D37" s="15" t="s">
         <v>395</v>
       </c>
       <c r="E37" t="s">
@@ -6500,7 +6270,7 @@
       <c r="C38" s="4" t="s">
         <v>554</v>
       </c>
-      <c r="D38" s="43" t="s">
+      <c r="D38" s="15" t="s">
         <v>395</v>
       </c>
       <c r="E38" t="s">
@@ -6520,7 +6290,7 @@
       <c r="C39" s="4" t="s">
         <v>1098</v>
       </c>
-      <c r="D39" s="43" t="s">
+      <c r="D39" s="15" t="s">
         <v>395</v>
       </c>
       <c r="E39" t="s">
@@ -6540,7 +6310,7 @@
       <c r="C40" s="4" t="s">
         <v>1278</v>
       </c>
-      <c r="D40" s="43" t="s">
+      <c r="D40" s="15" t="s">
         <v>395</v>
       </c>
       <c r="E40" t="s">
@@ -6560,7 +6330,7 @@
       <c r="C41" s="4" t="s">
         <v>577</v>
       </c>
-      <c r="D41" s="43" t="s">
+      <c r="D41" s="15" t="s">
         <v>578</v>
       </c>
       <c r="E41" s="2" t="s">
@@ -6581,7 +6351,7 @@
       <c r="C42" s="4" t="s">
         <v>1418</v>
       </c>
-      <c r="D42" s="43" t="s">
+      <c r="D42" s="15" t="s">
         <v>857</v>
       </c>
       <c r="E42" t="s">
@@ -6604,7 +6374,7 @@
       <c r="C43" s="4" t="s">
         <v>856</v>
       </c>
-      <c r="D43" s="43" t="s">
+      <c r="D43" s="15" t="s">
         <v>857</v>
       </c>
       <c r="E43" t="s">
@@ -6624,7 +6394,7 @@
       <c r="C44" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="D44" s="43" t="s">
+      <c r="D44" s="15" t="s">
         <v>319</v>
       </c>
       <c r="E44" t="s">
@@ -6644,7 +6414,7 @@
       <c r="C45" s="34" t="s">
         <v>321</v>
       </c>
-      <c r="D45" s="43" t="s">
+      <c r="D45" s="15" t="s">
         <v>319</v>
       </c>
       <c r="E45" t="s">
@@ -6665,7 +6435,7 @@
       <c r="C46" s="4" t="s">
         <v>1331</v>
       </c>
-      <c r="D46" s="43" t="s">
+      <c r="D46" s="15" t="s">
         <v>319</v>
       </c>
       <c r="E46" t="s">
@@ -6685,7 +6455,7 @@
       <c r="C47" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="D47" s="43" t="s">
+      <c r="D47" s="15" t="s">
         <v>436</v>
       </c>
       <c r="E47" t="s">
@@ -6705,7 +6475,7 @@
       <c r="C48" s="4" t="s">
         <v>566</v>
       </c>
-      <c r="D48" s="43" t="s">
+      <c r="D48" s="15" t="s">
         <v>436</v>
       </c>
       <c r="E48" t="s">
@@ -6725,7 +6495,7 @@
       <c r="C49" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D49" s="43" t="s">
+      <c r="D49" s="15" t="s">
         <v>83</v>
       </c>
       <c r="E49" t="s">
@@ -6745,7 +6515,7 @@
       <c r="C50" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D50" s="43" t="s">
+      <c r="D50" s="15" t="s">
         <v>36</v>
       </c>
       <c r="E50" s="5" t="s">
@@ -6765,7 +6535,7 @@
       <c r="C51" s="4" t="s">
         <v>614</v>
       </c>
-      <c r="D51" s="43" t="s">
+      <c r="D51" s="15" t="s">
         <v>36</v>
       </c>
       <c r="E51" s="5" t="s">
@@ -6787,7 +6557,7 @@
       <c r="C52" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D52" s="43" t="s">
+      <c r="D52" s="15" t="s">
         <v>36</v>
       </c>
       <c r="E52" t="s">
@@ -6807,7 +6577,7 @@
       <c r="C53" s="4" t="s">
         <v>408</v>
       </c>
-      <c r="D53" s="43" t="s">
+      <c r="D53" s="15" t="s">
         <v>409</v>
       </c>
       <c r="E53" t="s">
@@ -6827,7 +6597,7 @@
       <c r="C54" s="4" t="s">
         <v>1095</v>
       </c>
-      <c r="D54" s="43" t="s">
+      <c r="D54" s="15" t="s">
         <v>409</v>
       </c>
       <c r="E54" t="s">
@@ -6847,7 +6617,7 @@
       <c r="C55" s="4" t="s">
         <v>1023</v>
       </c>
-      <c r="D55" s="43" t="s">
+      <c r="D55" s="15" t="s">
         <v>1024</v>
       </c>
       <c r="E55" s="5" t="s">
@@ -6869,7 +6639,7 @@
       <c r="C56" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D56" s="43" t="s">
+      <c r="D56" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E56" t="s">
@@ -6889,7 +6659,7 @@
       <c r="C57" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="D57" s="43" t="s">
+      <c r="D57" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E57" t="s">
@@ -6909,7 +6679,7 @@
       <c r="C58" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="D58" s="43" t="s">
+      <c r="D58" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E58" t="s">
@@ -6929,7 +6699,7 @@
       <c r="C59" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="D59" s="43" t="s">
+      <c r="D59" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E59" t="s">
@@ -6949,7 +6719,7 @@
       <c r="C60" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="D60" s="43" t="s">
+      <c r="D60" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E60" t="s">
@@ -6969,7 +6739,7 @@
       <c r="C61" s="4" t="s">
         <v>528</v>
       </c>
-      <c r="D61" s="43" t="s">
+      <c r="D61" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E61" t="s">
@@ -6989,7 +6759,7 @@
       <c r="C62" s="4" t="s">
         <v>691</v>
       </c>
-      <c r="D62" s="43" t="s">
+      <c r="D62" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E62" t="s">
@@ -7009,7 +6779,7 @@
       <c r="C63" s="4" t="s">
         <v>990</v>
       </c>
-      <c r="D63" s="43" t="s">
+      <c r="D63" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E63" t="s">
@@ -7029,7 +6799,7 @@
       <c r="C64" s="4" t="s">
         <v>993</v>
       </c>
-      <c r="D64" s="43" t="s">
+      <c r="D64" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E64" t="s">
@@ -7049,7 +6819,7 @@
       <c r="C65" s="4" t="s">
         <v>1393</v>
       </c>
-      <c r="D65" s="43" t="s">
+      <c r="D65" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E65" t="s">
@@ -7069,7 +6839,7 @@
       <c r="C66" s="4" t="s">
         <v>557</v>
       </c>
-      <c r="D66" s="43" t="s">
+      <c r="D66" s="15" t="s">
         <v>558</v>
       </c>
       <c r="E66" t="s">
@@ -7089,7 +6859,7 @@
       <c r="C67" s="4" t="s">
         <v>328</v>
       </c>
-      <c r="D67" s="43" t="s">
+      <c r="D67" s="15" t="s">
         <v>329</v>
       </c>
       <c r="E67" t="s">
@@ -7109,7 +6879,7 @@
       <c r="C68" s="4" t="s">
         <v>949</v>
       </c>
-      <c r="D68" s="43" t="s">
+      <c r="D68" s="15" t="s">
         <v>329</v>
       </c>
       <c r="E68" t="s">
@@ -7129,7 +6899,7 @@
       <c r="C69" s="4" t="s">
         <v>1223</v>
       </c>
-      <c r="D69" s="43" t="s">
+      <c r="D69" s="15" t="s">
         <v>329</v>
       </c>
       <c r="E69" t="s">
@@ -7149,7 +6919,7 @@
       <c r="C70" s="4" t="s">
         <v>1289</v>
       </c>
-      <c r="D70" s="43" t="s">
+      <c r="D70" s="15" t="s">
         <v>329</v>
       </c>
       <c r="E70" t="s">
@@ -7169,7 +6939,7 @@
       <c r="C71" s="4" t="s">
         <v>750</v>
       </c>
-      <c r="D71" s="43" t="s">
+      <c r="D71" s="15" t="s">
         <v>751</v>
       </c>
       <c r="E71" t="s">
@@ -7189,7 +6959,7 @@
       <c r="C72" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="D72" s="43" t="s">
+      <c r="D72" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E72" s="5" t="s">
@@ -7211,7 +6981,7 @@
       <c r="C73" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="D73" s="43" t="s">
+      <c r="D73" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E73" s="5" t="s">
@@ -7233,7 +7003,7 @@
       <c r="C74" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="D74" s="43" t="s">
+      <c r="D74" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E74" s="5" t="s">
@@ -7255,7 +7025,7 @@
       <c r="C75" s="4" t="s">
         <v>682</v>
       </c>
-      <c r="D75" s="43" t="s">
+      <c r="D75" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E75" s="5" t="s">
@@ -7277,7 +7047,7 @@
       <c r="C76" s="4" t="s">
         <v>891</v>
       </c>
-      <c r="D76" s="43" t="s">
+      <c r="D76" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E76" s="5" t="s">
@@ -7299,7 +7069,7 @@
       <c r="C77" s="28" t="s">
         <v>965</v>
       </c>
-      <c r="D77" s="43" t="s">
+      <c r="D77" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E77" s="29" t="s">
@@ -7321,7 +7091,7 @@
       <c r="C78" s="4" t="s">
         <v>1169</v>
       </c>
-      <c r="D78" s="43" t="s">
+      <c r="D78" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E78" s="5" t="s">
@@ -7343,7 +7113,7 @@
       <c r="C79" s="4" t="s">
         <v>1240</v>
       </c>
-      <c r="D79" s="43" t="s">
+      <c r="D79" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E79" s="5" t="s">
@@ -7365,7 +7135,7 @@
       <c r="C80" s="4" t="s">
         <v>1378</v>
       </c>
-      <c r="D80" s="43" t="s">
+      <c r="D80" s="15" t="s">
         <v>274</v>
       </c>
       <c r="E80" s="5" t="s">
@@ -7387,7 +7157,7 @@
       <c r="C81" s="4" t="s">
         <v>1326</v>
       </c>
-      <c r="D81" s="43" t="s">
+      <c r="D81" s="15" t="s">
         <v>1327</v>
       </c>
       <c r="E81" t="s">
@@ -7407,7 +7177,7 @@
       <c r="C82" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D82" s="43" t="s">
+      <c r="D82" s="15" t="s">
         <v>88</v>
       </c>
       <c r="E82" s="5" t="s">
@@ -7418,14 +7188,16 @@
       </c>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A83" s="28"/>
+      <c r="A83" s="28" t="s">
+        <v>1556</v>
+      </c>
       <c r="B83" s="28" t="s">
         <v>99</v>
       </c>
       <c r="C83" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="D83" s="43" t="s">
+      <c r="D83" s="15" t="s">
         <v>101</v>
       </c>
       <c r="E83" s="29" t="s">
@@ -7445,7 +7217,7 @@
       <c r="C84" s="4" t="s">
         <v>464</v>
       </c>
-      <c r="D84" s="43" t="s">
+      <c r="D84" s="15" t="s">
         <v>465</v>
       </c>
       <c r="E84" s="2" t="s">
@@ -7467,7 +7239,7 @@
       <c r="C85" s="4" t="s">
         <v>524</v>
       </c>
-      <c r="D85" s="43" t="s">
+      <c r="D85" s="15" t="s">
         <v>525</v>
       </c>
       <c r="E85" s="5" t="s">
@@ -7487,7 +7259,7 @@
       <c r="C86" s="4" t="s">
         <v>894</v>
       </c>
-      <c r="D86" s="43" t="s">
+      <c r="D86" s="15" t="s">
         <v>525</v>
       </c>
       <c r="E86" s="5" t="s">
@@ -7509,7 +7281,7 @@
       <c r="C87" s="4" t="s">
         <v>617</v>
       </c>
-      <c r="D87" s="43" t="s">
+      <c r="D87" s="15" t="s">
         <v>618</v>
       </c>
       <c r="E87" s="2" t="s">
@@ -7529,7 +7301,7 @@
       <c r="C88" s="4" t="s">
         <v>839</v>
       </c>
-      <c r="D88" s="43" t="s">
+      <c r="D88" s="15" t="s">
         <v>618</v>
       </c>
       <c r="E88" s="2" t="s">
@@ -7549,7 +7321,7 @@
       <c r="C89" s="4" t="s">
         <v>983</v>
       </c>
-      <c r="D89" s="43" t="s">
+      <c r="D89" s="15" t="s">
         <v>984</v>
       </c>
       <c r="E89" s="2" t="s">
@@ -7569,7 +7341,7 @@
       <c r="C90" s="4" t="s">
         <v>1001</v>
       </c>
-      <c r="D90" s="43" t="s">
+      <c r="D90" s="15" t="s">
         <v>984</v>
       </c>
       <c r="E90" s="2" t="s">
@@ -7589,7 +7361,7 @@
       <c r="C91" s="4" t="s">
         <v>1060</v>
       </c>
-      <c r="D91" s="43" t="s">
+      <c r="D91" s="15" t="s">
         <v>1061</v>
       </c>
       <c r="E91" s="2" t="s">
@@ -7609,7 +7381,7 @@
       <c r="C92" s="4" t="s">
         <v>609</v>
       </c>
-      <c r="D92" s="43" t="s">
+      <c r="D92" s="15" t="s">
         <v>610</v>
       </c>
       <c r="E92" s="5" t="s">
@@ -7622,14 +7394,16 @@
       <c r="O92" s="5"/>
     </row>
     <row r="93" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A93" s="28"/>
+      <c r="A93" s="28" t="s">
+        <v>1557</v>
+      </c>
       <c r="B93" s="28" t="s">
         <v>1076</v>
       </c>
       <c r="C93" s="28" t="s">
         <v>1077</v>
       </c>
-      <c r="D93" s="43" t="s">
+      <c r="D93" s="15" t="s">
         <v>610</v>
       </c>
       <c r="E93" s="29" t="s">
@@ -7651,7 +7425,7 @@
       <c r="C94" s="4" t="s">
         <v>733</v>
       </c>
-      <c r="D94" s="43" t="s">
+      <c r="D94" s="15" t="s">
         <v>734</v>
       </c>
       <c r="E94" s="5" t="s">
@@ -7671,7 +7445,7 @@
       <c r="C95" s="4" t="s">
         <v>755</v>
       </c>
-      <c r="D95" s="43" t="s">
+      <c r="D95" s="15" t="s">
         <v>734</v>
       </c>
       <c r="E95" s="5" t="s">
@@ -7693,7 +7467,7 @@
       <c r="C96" s="4" t="s">
         <v>766</v>
       </c>
-      <c r="D96" s="43" t="s">
+      <c r="D96" s="15" t="s">
         <v>734</v>
       </c>
       <c r="E96" s="5" t="s">
@@ -7715,7 +7489,7 @@
       <c r="C97" s="4" t="s">
         <v>955</v>
       </c>
-      <c r="D97" s="43" t="s">
+      <c r="D97" s="15" t="s">
         <v>956</v>
       </c>
       <c r="E97" s="5" t="s">
@@ -7737,7 +7511,7 @@
       <c r="C98" s="4" t="s">
         <v>834</v>
       </c>
-      <c r="D98" s="43" t="s">
+      <c r="D98" s="15" t="s">
         <v>835</v>
       </c>
       <c r="E98" s="5" t="s">
@@ -7759,7 +7533,7 @@
       <c r="C99" s="4" t="s">
         <v>1342</v>
       </c>
-      <c r="D99" s="43" t="s">
+      <c r="D99" s="15" t="s">
         <v>1343</v>
       </c>
       <c r="E99" s="5" t="s">
@@ -7781,7 +7555,7 @@
       <c r="C100" s="4" t="s">
         <v>1447</v>
       </c>
-      <c r="D100" s="43" t="s">
+      <c r="D100" s="15" t="s">
         <v>1343</v>
       </c>
       <c r="E100" s="5" t="s">
@@ -7803,7 +7577,7 @@
       <c r="C101" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D101" s="43" t="s">
+      <c r="D101" s="15" t="s">
         <v>55</v>
       </c>
       <c r="E101" s="5" t="s">
@@ -7825,7 +7599,7 @@
       <c r="C102" s="4" t="s">
         <v>1258</v>
       </c>
-      <c r="D102" s="43" t="s">
+      <c r="D102" s="15" t="s">
         <v>55</v>
       </c>
       <c r="E102" s="5" t="s">
@@ -7847,7 +7621,7 @@
       <c r="C103" s="4" t="s">
         <v>919</v>
       </c>
-      <c r="D103" s="43" t="s">
+      <c r="D103" s="15" t="s">
         <v>920</v>
       </c>
       <c r="E103" s="5" t="s">
@@ -7869,7 +7643,7 @@
       <c r="C104" s="4" t="s">
         <v>921</v>
       </c>
-      <c r="D104" s="43" t="s">
+      <c r="D104" s="15" t="s">
         <v>920</v>
       </c>
       <c r="E104" s="5" t="s">
@@ -7891,7 +7665,7 @@
       <c r="C105" s="4" t="s">
         <v>1107</v>
       </c>
-      <c r="D105" s="43" t="s">
+      <c r="D105" s="15" t="s">
         <v>1108</v>
       </c>
       <c r="E105" s="5" t="s">
@@ -7913,7 +7687,7 @@
       <c r="C106" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D106" s="43" t="s">
+      <c r="D106" s="15" t="s">
         <v>59</v>
       </c>
       <c r="E106" s="5" t="s">
@@ -7935,7 +7709,7 @@
       <c r="C107" s="4" t="s">
         <v>1266</v>
       </c>
-      <c r="D107" s="43" t="s">
+      <c r="D107" s="15" t="s">
         <v>1267</v>
       </c>
       <c r="E107" s="5" t="s">
@@ -7957,7 +7731,7 @@
       <c r="C108" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="D108" s="43" t="s">
+      <c r="D108" s="15" t="s">
         <v>293</v>
       </c>
       <c r="E108" s="5" t="s">
@@ -7979,7 +7753,7 @@
       <c r="C109" s="4" t="s">
         <v>1004</v>
       </c>
-      <c r="D109" s="43" t="s">
+      <c r="D109" s="15" t="s">
         <v>1005</v>
       </c>
       <c r="E109" s="5" t="s">
@@ -8001,7 +7775,7 @@
       <c r="C110" s="4" t="s">
         <v>456</v>
       </c>
-      <c r="D110" s="43" t="s">
+      <c r="D110" s="15" t="s">
         <v>457</v>
       </c>
       <c r="E110" s="5" t="s">
@@ -8023,7 +7797,7 @@
       <c r="C111" s="4" t="s">
         <v>551</v>
       </c>
-      <c r="D111" s="43" t="s">
+      <c r="D111" s="15" t="s">
         <v>457</v>
       </c>
       <c r="E111" s="5" t="s">
@@ -8045,7 +7819,7 @@
       <c r="C112" s="4" t="s">
         <v>884</v>
       </c>
-      <c r="D112" s="43" t="s">
+      <c r="D112" s="15" t="s">
         <v>457</v>
       </c>
       <c r="E112" s="5" t="s">
@@ -8067,7 +7841,7 @@
       <c r="C113" s="4" t="s">
         <v>1075</v>
       </c>
-      <c r="D113" s="43" t="s">
+      <c r="D113" s="15" t="s">
         <v>457</v>
       </c>
       <c r="E113" s="5" t="s">
@@ -8089,7 +7863,7 @@
       <c r="C114" s="4" t="s">
         <v>447</v>
       </c>
-      <c r="D114" s="43" t="s">
+      <c r="D114" s="15" t="s">
         <v>448</v>
       </c>
       <c r="E114" s="5" t="s">
@@ -8111,7 +7885,7 @@
       <c r="C115" s="4" t="s">
         <v>497</v>
       </c>
-      <c r="D115" s="43" t="s">
+      <c r="D115" s="15" t="s">
         <v>448</v>
       </c>
       <c r="E115" s="5" t="s">
@@ -8133,7 +7907,7 @@
       <c r="C116" s="4" t="s">
         <v>1207</v>
       </c>
-      <c r="D116" s="43" t="s">
+      <c r="D116" s="15" t="s">
         <v>448</v>
       </c>
       <c r="E116" s="5" t="s">
@@ -8155,7 +7929,7 @@
       <c r="C117" s="4" t="s">
         <v>600</v>
       </c>
-      <c r="D117" s="43" t="s">
+      <c r="D117" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E117" s="5" t="s">
@@ -8180,7 +7954,7 @@
       <c r="C118" s="4" t="s">
         <v>717</v>
       </c>
-      <c r="D118" s="43" t="s">
+      <c r="D118" s="15" t="s">
         <v>718</v>
       </c>
       <c r="E118" s="2" t="s">
@@ -8200,7 +7974,7 @@
       <c r="C119" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="D119" s="43" t="s">
+      <c r="D119" s="15" t="s">
         <v>143</v>
       </c>
       <c r="E119" s="5" t="s">
@@ -8222,7 +7996,7 @@
       <c r="C120" s="4" t="s">
         <v>346</v>
       </c>
-      <c r="D120" s="43" t="s">
+      <c r="D120" s="15" t="s">
         <v>143</v>
       </c>
       <c r="E120" s="5" t="s">
@@ -8244,7 +8018,7 @@
       <c r="C121" s="4" t="s">
         <v>1127</v>
       </c>
-      <c r="D121" s="43" t="s">
+      <c r="D121" s="15" t="s">
         <v>143</v>
       </c>
       <c r="E121" s="5" t="s">
@@ -8266,7 +8040,7 @@
       <c r="C122" s="4" t="s">
         <v>1296</v>
       </c>
-      <c r="D122" s="43" t="s">
+      <c r="D122" s="15" t="s">
         <v>1297</v>
       </c>
       <c r="E122" s="5" t="s">
@@ -8279,14 +8053,16 @@
       <c r="O122" s="5"/>
     </row>
     <row r="123" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A123" s="28"/>
+      <c r="A123" s="28" t="s">
+        <v>1558</v>
+      </c>
       <c r="B123" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C123" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="D123" s="43" t="s">
+      <c r="D123" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E123" s="29" t="s">
@@ -8295,7 +8071,6 @@
       <c r="F123" t="s">
         <v>18</v>
       </c>
-      <c r="G123" s="49"/>
       <c r="N123" s="7"/>
       <c r="O123" s="5"/>
     </row>
@@ -8309,7 +8084,7 @@
       <c r="C124" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D124" s="43" t="s">
+      <c r="D124" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E124" s="5" t="s">
@@ -8331,7 +8106,7 @@
       <c r="C125" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D125" s="43" t="s">
+      <c r="D125" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E125" s="5" t="s">
@@ -8353,7 +8128,7 @@
       <c r="C126" s="4" t="s">
         <v>418</v>
       </c>
-      <c r="D126" s="43" t="s">
+      <c r="D126" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E126" s="5" t="s">
@@ -8376,7 +8151,7 @@
       <c r="C127" s="34" t="s">
         <v>419</v>
       </c>
-      <c r="D127" s="43" t="s">
+      <c r="D127" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E127" s="5" t="s">
@@ -8390,14 +8165,16 @@
       </c>
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A128" s="28"/>
+      <c r="A128" s="28" t="s">
+        <v>1559</v>
+      </c>
       <c r="B128" s="28" t="s">
         <v>767</v>
       </c>
       <c r="C128" s="28" t="s">
         <v>768</v>
       </c>
-      <c r="D128" s="43" t="s">
+      <c r="D128" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E128" s="29" t="s">
@@ -8410,14 +8187,16 @@
       <c r="O128" s="5"/>
     </row>
     <row r="129" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A129" s="28"/>
+      <c r="A129" s="28" t="s">
+        <v>1560</v>
+      </c>
       <c r="B129" s="28" t="s">
         <v>789</v>
       </c>
       <c r="C129" s="28" t="s">
         <v>790</v>
       </c>
-      <c r="D129" s="43" t="s">
+      <c r="D129" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E129" s="29" t="s">
@@ -8439,7 +8218,7 @@
       <c r="C130" s="4" t="s">
         <v>708</v>
       </c>
-      <c r="D130" s="44" t="s">
+      <c r="D130" s="43" t="s">
         <v>709</v>
       </c>
       <c r="E130" s="34" t="s">
@@ -8462,7 +8241,7 @@
       <c r="C131" s="34" t="s">
         <v>1038</v>
       </c>
-      <c r="D131" s="44" t="s">
+      <c r="D131" s="43" t="s">
         <v>709</v>
       </c>
       <c r="E131" s="34" t="s">
@@ -8482,7 +8261,7 @@
       <c r="C132" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D132" s="43" t="s">
+      <c r="D132" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E132" s="2" t="s">
@@ -8491,20 +8270,20 @@
       <c r="F132" t="s">
         <v>18</v>
       </c>
-      <c r="G132" s="49"/>
-      <c r="I132" s="49"/>
       <c r="N132" s="7"/>
       <c r="O132" s="2"/>
     </row>
     <row r="133" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A133" s="28"/>
+      <c r="A133" s="28" t="s">
+        <v>1561</v>
+      </c>
       <c r="B133" s="28" t="s">
         <v>174</v>
       </c>
       <c r="C133" s="28" t="s">
         <v>175</v>
       </c>
-      <c r="D133" s="43" t="s">
+      <c r="D133" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E133" s="30" t="s">
@@ -8513,8 +8292,6 @@
       <c r="F133" t="s">
         <v>18</v>
       </c>
-      <c r="G133" s="49"/>
-      <c r="I133" s="49"/>
     </row>
     <row r="134" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A134" s="4" t="s">
@@ -8526,7 +8303,7 @@
       <c r="C134" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="D134" s="43" t="s">
+      <c r="D134" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E134" s="2" t="s">
@@ -8535,18 +8312,18 @@
       <c r="F134" t="s">
         <v>18</v>
       </c>
-      <c r="G134" s="49"/>
-      <c r="I134" s="49"/>
     </row>
     <row r="135" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A135" s="28"/>
+      <c r="A135" s="28" t="s">
+        <v>1562</v>
+      </c>
       <c r="B135" s="28" t="s">
         <v>288</v>
       </c>
       <c r="C135" s="28" t="s">
         <v>289</v>
       </c>
-      <c r="D135" s="43" t="s">
+      <c r="D135" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E135" s="30" t="s">
@@ -8555,8 +8332,6 @@
       <c r="F135" t="s">
         <v>18</v>
       </c>
-      <c r="G135" s="49"/>
-      <c r="I135" s="49"/>
     </row>
     <row r="136" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
@@ -8568,7 +8343,7 @@
       <c r="C136" s="4" t="s">
         <v>603</v>
       </c>
-      <c r="D136" s="43" t="s">
+      <c r="D136" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E136" s="2" t="s">
@@ -8577,8 +8352,6 @@
       <c r="F136" t="s">
         <v>18</v>
       </c>
-      <c r="G136" s="49"/>
-      <c r="I136" s="49"/>
     </row>
     <row r="137" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
@@ -8590,7 +8363,7 @@
       <c r="C137" s="4" t="s">
         <v>606</v>
       </c>
-      <c r="D137" s="43" t="s">
+      <c r="D137" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E137" s="2" t="s">
@@ -8599,8 +8372,6 @@
       <c r="F137" t="s">
         <v>18</v>
       </c>
-      <c r="G137" s="49"/>
-      <c r="I137" s="49"/>
     </row>
     <row r="138" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A138" s="4" t="s">
@@ -8612,7 +8383,7 @@
       <c r="C138" s="4" t="s">
         <v>780</v>
       </c>
-      <c r="D138" s="43" t="s">
+      <c r="D138" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E138" s="2" t="s">
@@ -8621,8 +8392,6 @@
       <c r="F138" t="s">
         <v>18</v>
       </c>
-      <c r="G138" s="49"/>
-      <c r="I138" s="49"/>
     </row>
     <row r="139" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
@@ -8634,7 +8403,7 @@
       <c r="C139" s="4" t="s">
         <v>793</v>
       </c>
-      <c r="D139" s="43" t="s">
+      <c r="D139" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E139" s="2" t="s">
@@ -8643,8 +8412,6 @@
       <c r="F139" t="s">
         <v>18</v>
       </c>
-      <c r="G139" s="49"/>
-      <c r="I139" s="49"/>
     </row>
     <row r="140" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A140" s="4" t="s">
@@ -8656,7 +8423,7 @@
       <c r="C140" s="4" t="s">
         <v>796</v>
       </c>
-      <c r="D140" s="43" t="s">
+      <c r="D140" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E140" s="2" t="s">
@@ -8665,8 +8432,6 @@
       <c r="F140" t="s">
         <v>18</v>
       </c>
-      <c r="G140" s="49"/>
-      <c r="I140" s="49"/>
       <c r="N140" s="7"/>
       <c r="O140" s="5"/>
     </row>
@@ -8680,7 +8445,7 @@
       <c r="C141" s="4" t="s">
         <v>853</v>
       </c>
-      <c r="D141" s="43" t="s">
+      <c r="D141" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E141" s="2" t="s">
@@ -8689,8 +8454,6 @@
       <c r="F141" t="s">
         <v>18</v>
       </c>
-      <c r="G141" s="49"/>
-      <c r="I141" s="49"/>
       <c r="N141" s="7"/>
       <c r="O141" s="5"/>
     </row>
@@ -8704,7 +8467,7 @@
       <c r="C142" s="4" t="s">
         <v>941</v>
       </c>
-      <c r="D142" s="43" t="s">
+      <c r="D142" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E142" s="2" t="s">
@@ -8713,8 +8476,6 @@
       <c r="F142" t="s">
         <v>18</v>
       </c>
-      <c r="G142" s="49"/>
-      <c r="I142" s="49"/>
     </row>
     <row r="143" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A143" s="4" t="s">
@@ -8726,7 +8487,7 @@
       <c r="C143" s="4" t="s">
         <v>952</v>
       </c>
-      <c r="D143" s="43" t="s">
+      <c r="D143" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E143" s="2" t="s">
@@ -8735,8 +8496,6 @@
       <c r="F143" t="s">
         <v>18</v>
       </c>
-      <c r="G143" s="49"/>
-      <c r="I143" s="49"/>
     </row>
     <row r="144" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A144" s="4" t="s">
@@ -8748,7 +8507,7 @@
       <c r="C144" s="4" t="s">
         <v>972</v>
       </c>
-      <c r="D144" s="43" t="s">
+      <c r="D144" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E144" s="2" t="s">
@@ -8757,8 +8516,6 @@
       <c r="F144" t="s">
         <v>18</v>
       </c>
-      <c r="G144" s="49"/>
-      <c r="I144" s="49"/>
       <c r="N144" s="7"/>
       <c r="O144" s="2"/>
     </row>
@@ -8772,7 +8529,7 @@
       <c r="C145" s="4" t="s">
         <v>999</v>
       </c>
-      <c r="D145" s="43" t="s">
+      <c r="D145" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E145" s="2" t="s">
@@ -8781,8 +8538,6 @@
       <c r="F145" t="s">
         <v>18</v>
       </c>
-      <c r="G145" s="49"/>
-      <c r="I145" s="49"/>
     </row>
     <row r="146" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A146" s="4" t="s">
@@ -8794,7 +8549,7 @@
       <c r="C146" s="4" t="s">
         <v>1089</v>
       </c>
-      <c r="D146" s="43" t="s">
+      <c r="D146" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E146" s="2" t="s">
@@ -8803,8 +8558,6 @@
       <c r="F146" t="s">
         <v>18</v>
       </c>
-      <c r="G146" s="49"/>
-      <c r="I146" s="49"/>
     </row>
     <row r="147" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A147" s="4" t="s">
@@ -8816,7 +8569,7 @@
       <c r="C147" s="4" t="s">
         <v>1444</v>
       </c>
-      <c r="D147" s="43" t="s">
+      <c r="D147" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E147" s="2" t="s">
@@ -8825,8 +8578,6 @@
       <c r="F147" t="s">
         <v>18</v>
       </c>
-      <c r="G147" s="49"/>
-      <c r="I147" s="49"/>
     </row>
     <row r="148" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A148" s="4" t="s">
@@ -8838,7 +8589,7 @@
       <c r="C148" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="D148" s="43" t="s">
+      <c r="D148" s="15" t="s">
         <v>31</v>
       </c>
       <c r="E148" s="2" t="s">
@@ -8847,8 +8598,6 @@
       <c r="F148" t="s">
         <v>18</v>
       </c>
-      <c r="G148" s="49"/>
-      <c r="I148" s="49"/>
       <c r="N148" s="7"/>
       <c r="O148" s="2"/>
     </row>
@@ -8862,7 +8611,7 @@
       <c r="C149" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D149" s="43" t="s">
+      <c r="D149" s="15" t="s">
         <v>31</v>
       </c>
       <c r="E149" s="2" t="s">
@@ -8871,8 +8620,6 @@
       <c r="F149" t="s">
         <v>18</v>
       </c>
-      <c r="G149" s="49"/>
-      <c r="I149" s="49"/>
       <c r="N149" s="7"/>
       <c r="O149" s="2"/>
     </row>
@@ -8886,7 +8633,7 @@
       <c r="C150" s="4" t="s">
         <v>811</v>
       </c>
-      <c r="D150" s="43" t="s">
+      <c r="D150" s="15" t="s">
         <v>31</v>
       </c>
       <c r="E150" s="2" t="s">
@@ -8895,8 +8642,6 @@
       <c r="F150" t="s">
         <v>18</v>
       </c>
-      <c r="G150" s="49"/>
-      <c r="I150" s="49"/>
       <c r="N150" s="7"/>
       <c r="O150" s="5"/>
     </row>
@@ -8910,7 +8655,7 @@
       <c r="C151" s="4" t="s">
         <v>1028</v>
       </c>
-      <c r="D151" s="43" t="s">
+      <c r="D151" s="15" t="s">
         <v>31</v>
       </c>
       <c r="E151" s="2" t="s">
@@ -8919,8 +8664,6 @@
       <c r="F151" t="s">
         <v>18</v>
       </c>
-      <c r="G151" s="49"/>
-      <c r="I151" s="49"/>
       <c r="N151" s="7"/>
       <c r="O151" s="5"/>
     </row>
@@ -8934,7 +8677,7 @@
       <c r="C152" s="4" t="s">
         <v>1057</v>
       </c>
-      <c r="D152" s="43" t="s">
+      <c r="D152" s="15" t="s">
         <v>31</v>
       </c>
       <c r="E152" s="2" t="s">
@@ -8943,8 +8686,6 @@
       <c r="F152" t="s">
         <v>18</v>
       </c>
-      <c r="G152" s="49"/>
-      <c r="I152" s="49"/>
       <c r="N152" s="7"/>
       <c r="O152" s="2"/>
     </row>
@@ -8958,7 +8699,7 @@
       <c r="C153" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="D153" s="43" t="s">
+      <c r="D153" s="15" t="s">
         <v>246</v>
       </c>
       <c r="E153" s="2" t="s">
@@ -8967,8 +8708,8 @@
       <c r="F153" t="s">
         <v>18</v>
       </c>
-      <c r="G153" s="43"/>
-      <c r="I153" s="50"/>
+      <c r="G153" s="15"/>
+      <c r="I153" s="2"/>
       <c r="N153" s="7"/>
       <c r="O153" s="5"/>
     </row>
@@ -8982,7 +8723,7 @@
       <c r="C154" s="4" t="s">
         <v>300</v>
       </c>
-      <c r="D154" s="43" t="s">
+      <c r="D154" s="15" t="s">
         <v>301</v>
       </c>
       <c r="E154" s="5" t="s">
@@ -8991,8 +8732,6 @@
       <c r="F154" t="s">
         <v>18</v>
       </c>
-      <c r="G154" s="49"/>
-      <c r="I154" s="49"/>
       <c r="N154" s="7"/>
       <c r="O154" s="2"/>
     </row>
@@ -9006,7 +8745,7 @@
       <c r="C155" s="4" t="s">
         <v>646</v>
       </c>
-      <c r="D155" s="43" t="s">
+      <c r="D155" s="15" t="s">
         <v>647</v>
       </c>
       <c r="E155" s="2" t="s">
@@ -9015,8 +8754,6 @@
       <c r="F155" t="s">
         <v>18</v>
       </c>
-      <c r="G155" s="49"/>
-      <c r="I155" s="49"/>
       <c r="N155" s="7"/>
       <c r="O155" s="5"/>
     </row>
@@ -9030,7 +8767,7 @@
       <c r="C156" s="4" t="s">
         <v>1064</v>
       </c>
-      <c r="D156" s="44" t="s">
+      <c r="D156" s="43" t="s">
         <v>1065</v>
       </c>
       <c r="E156" s="34" t="s">
@@ -9039,7 +8776,7 @@
       <c r="F156" t="s">
         <v>18</v>
       </c>
-      <c r="G156" s="51" t="s">
+      <c r="G156" s="39" t="s">
         <v>1067</v>
       </c>
       <c r="N156" s="7"/>
@@ -9055,7 +8792,7 @@
       <c r="C157" s="34" t="s">
         <v>1068</v>
       </c>
-      <c r="D157" s="44" t="s">
+      <c r="D157" s="43" t="s">
         <v>1065</v>
       </c>
       <c r="E157" s="34" t="s">
@@ -9073,7 +8810,7 @@
       <c r="C158" s="4" t="s">
         <v>1405</v>
       </c>
-      <c r="D158" s="43" t="s">
+      <c r="D158" s="15" t="s">
         <v>1406</v>
       </c>
       <c r="E158" s="5" t="s">
@@ -9095,7 +8832,7 @@
       <c r="C159" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="D159" s="43" t="s">
+      <c r="D159" s="15" t="s">
         <v>172</v>
       </c>
       <c r="E159" s="5" t="s">
@@ -9117,7 +8854,7 @@
       <c r="C160" s="34" t="s">
         <v>725</v>
       </c>
-      <c r="D160" s="44" t="s">
+      <c r="D160" s="43" t="s">
         <v>726</v>
       </c>
       <c r="E160" s="34" t="s">
@@ -9135,7 +8872,7 @@
       <c r="C161" s="4" t="s">
         <v>1270</v>
       </c>
-      <c r="D161" s="43" t="s">
+      <c r="D161" s="15" t="s">
         <v>1271</v>
       </c>
       <c r="E161" s="5" t="s">
@@ -9157,7 +8894,7 @@
       <c r="C162" s="4" t="s">
         <v>1009</v>
       </c>
-      <c r="D162" s="43" t="s">
+      <c r="D162" s="15" t="s">
         <v>1010</v>
       </c>
       <c r="E162" s="2" t="s">
@@ -9179,7 +8916,7 @@
       <c r="C163" s="4" t="s">
         <v>771</v>
       </c>
-      <c r="D163" s="43" t="s">
+      <c r="D163" s="15" t="s">
         <v>772</v>
       </c>
       <c r="E163" s="5" t="s">
@@ -9201,7 +8938,7 @@
       <c r="C164" s="21" t="s">
         <v>1122</v>
       </c>
-      <c r="D164" s="43" t="s">
+      <c r="D164" s="15" t="s">
         <v>1123</v>
       </c>
       <c r="E164" s="28" t="s">
@@ -9223,7 +8960,7 @@
       <c r="C165" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="D165" s="43" t="s">
+      <c r="D165" s="15" t="s">
         <v>227</v>
       </c>
       <c r="E165" t="s">
@@ -9243,7 +8980,7 @@
       <c r="C166" s="4" t="s">
         <v>461</v>
       </c>
-      <c r="D166" s="43" t="s">
+      <c r="D166" s="15" t="s">
         <v>227</v>
       </c>
       <c r="E166" t="s">
@@ -9263,7 +9000,7 @@
       <c r="C167" s="4" t="s">
         <v>1179</v>
       </c>
-      <c r="D167" s="43" t="s">
+      <c r="D167" s="15" t="s">
         <v>227</v>
       </c>
       <c r="E167" t="s">
@@ -9283,7 +9020,7 @@
       <c r="C168" s="4" t="s">
         <v>1319</v>
       </c>
-      <c r="D168" s="43" t="s">
+      <c r="D168" s="15" t="s">
         <v>227</v>
       </c>
       <c r="E168" s="5" t="s">
@@ -9305,7 +9042,7 @@
       <c r="C169" s="4" t="s">
         <v>1080</v>
       </c>
-      <c r="D169" s="43" t="s">
+      <c r="D169" s="15" t="s">
         <v>1081</v>
       </c>
       <c r="E169" s="5" t="s">
@@ -9327,7 +9064,7 @@
       <c r="C170" s="4" t="s">
         <v>657</v>
       </c>
-      <c r="D170" s="43" t="s">
+      <c r="D170" s="15" t="s">
         <v>658</v>
       </c>
       <c r="E170" s="5" t="s">
@@ -9349,7 +9086,7 @@
       <c r="C171" s="34" t="s">
         <v>660</v>
       </c>
-      <c r="D171" s="43" t="s">
+      <c r="D171" s="15" t="s">
         <v>658</v>
       </c>
       <c r="E171" s="5" t="s">
@@ -9370,7 +9107,7 @@
       <c r="C172" s="34" t="s">
         <v>910</v>
       </c>
-      <c r="D172" s="43" t="s">
+      <c r="D172" s="15" t="s">
         <v>658</v>
       </c>
       <c r="E172" s="5" t="s">
@@ -9391,7 +9128,7 @@
       <c r="C173" s="4" t="s">
         <v>912</v>
       </c>
-      <c r="D173" s="43" t="s">
+      <c r="D173" s="15" t="s">
         <v>658</v>
       </c>
       <c r="E173" s="5" t="s">
@@ -9413,7 +9150,7 @@
       <c r="C174" s="4" t="s">
         <v>962</v>
       </c>
-      <c r="D174" s="43" t="s">
+      <c r="D174" s="15" t="s">
         <v>658</v>
       </c>
       <c r="E174" s="5" t="s">
@@ -9435,7 +9172,7 @@
       <c r="C175" s="4" t="s">
         <v>1092</v>
       </c>
-      <c r="D175" s="43" t="s">
+      <c r="D175" s="15" t="s">
         <v>658</v>
       </c>
       <c r="E175" s="5" t="s">
@@ -9457,7 +9194,7 @@
       <c r="C176" s="34" t="s">
         <v>1218</v>
       </c>
-      <c r="D176" s="43" t="s">
+      <c r="D176" s="15" t="s">
         <v>658</v>
       </c>
       <c r="E176" s="5" t="s">
@@ -9478,7 +9215,7 @@
       <c r="C177" s="4" t="s">
         <v>1220</v>
       </c>
-      <c r="D177" s="43" t="s">
+      <c r="D177" s="15" t="s">
         <v>658</v>
       </c>
       <c r="E177" s="5" t="s">
@@ -9500,7 +9237,7 @@
       <c r="C178" s="4" t="s">
         <v>944</v>
       </c>
-      <c r="D178" s="43" t="s">
+      <c r="D178" s="15" t="s">
         <v>945</v>
       </c>
       <c r="E178" s="5" t="s">
@@ -9522,7 +9259,7 @@
       <c r="C179" s="4" t="s">
         <v>1347</v>
       </c>
-      <c r="D179" s="43" t="s">
+      <c r="D179" s="15" t="s">
         <v>945</v>
       </c>
       <c r="E179" s="5" t="s">
@@ -9542,7 +9279,7 @@
       <c r="C180" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="D180" s="43" t="s">
+      <c r="D180" s="15" t="s">
         <v>364</v>
       </c>
       <c r="E180" s="2" t="s">
@@ -9555,14 +9292,16 @@
       <c r="O180" s="5"/>
     </row>
     <row r="181" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A181" s="28"/>
+      <c r="A181" s="28" t="s">
+        <v>1563</v>
+      </c>
       <c r="B181" s="28" t="s">
         <v>977</v>
       </c>
       <c r="C181" s="28" t="s">
         <v>978</v>
       </c>
-      <c r="D181" s="43" t="s">
+      <c r="D181" s="15" t="s">
         <v>979</v>
       </c>
       <c r="E181" s="29" t="s">
@@ -9575,14 +9314,16 @@
       <c r="O181" s="5"/>
     </row>
     <row r="182" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A182" s="28"/>
+      <c r="A182" s="28" t="s">
+        <v>1564</v>
+      </c>
       <c r="B182" s="28" t="s">
         <v>973</v>
       </c>
       <c r="C182" s="28" t="s">
         <v>974</v>
       </c>
-      <c r="D182" s="43" t="s">
+      <c r="D182" s="15" t="s">
         <v>975</v>
       </c>
       <c r="E182" s="29" t="s">
@@ -9604,7 +9345,7 @@
       <c r="C183" s="4" t="s">
         <v>821</v>
       </c>
-      <c r="D183" s="43" t="s">
+      <c r="D183" s="15" t="s">
         <v>822</v>
       </c>
       <c r="E183" s="5" t="s">
@@ -9626,7 +9367,7 @@
       <c r="C184" s="4" t="s">
         <v>924</v>
       </c>
-      <c r="D184" s="43" t="s">
+      <c r="D184" s="15" t="s">
         <v>822</v>
       </c>
       <c r="E184" s="5" t="s">
@@ -9648,7 +9389,7 @@
       <c r="C185" s="4" t="s">
         <v>1334</v>
       </c>
-      <c r="D185" s="43" t="s">
+      <c r="D185" s="15" t="s">
         <v>1335</v>
       </c>
       <c r="E185" s="2" t="s">
@@ -9670,7 +9411,7 @@
       <c r="C186" s="34" t="s">
         <v>250</v>
       </c>
-      <c r="D186" s="43" t="s">
+      <c r="D186" s="15" t="s">
         <v>251</v>
       </c>
       <c r="E186" s="2" t="s">
@@ -9691,7 +9432,7 @@
       <c r="C187" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="D187" s="43" t="s">
+      <c r="D187" s="15" t="s">
         <v>251</v>
       </c>
       <c r="E187" s="41" t="s">
@@ -9713,7 +9454,7 @@
       <c r="C188" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="D188" s="43" t="s">
+      <c r="D188" s="15" t="s">
         <v>251</v>
       </c>
       <c r="E188" s="2" t="s">
@@ -9735,7 +9476,7 @@
       <c r="C189" s="4" t="s">
         <v>702</v>
       </c>
-      <c r="D189" s="43" t="s">
+      <c r="D189" s="15" t="s">
         <v>251</v>
       </c>
       <c r="E189" s="2" t="s">
@@ -9757,7 +9498,7 @@
       <c r="C190" s="4" t="s">
         <v>1462</v>
       </c>
-      <c r="D190" s="43" t="s">
+      <c r="D190" s="15" t="s">
         <v>251</v>
       </c>
       <c r="E190" s="2" t="s">
@@ -9779,7 +9520,7 @@
       <c r="C191" s="4" t="s">
         <v>1462</v>
       </c>
-      <c r="D191" s="43" t="s">
+      <c r="D191" s="15" t="s">
         <v>251</v>
       </c>
       <c r="E191" s="2" t="s">
@@ -9801,7 +9542,7 @@
       <c r="C192" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="D192" s="43" t="s">
+      <c r="D192" s="15" t="s">
         <v>382</v>
       </c>
       <c r="E192" s="2" t="s">
@@ -9823,7 +9564,7 @@
       <c r="C193" s="34" t="s">
         <v>1360</v>
       </c>
-      <c r="D193" s="44" t="s">
+      <c r="D193" s="43" t="s">
         <v>1361</v>
       </c>
       <c r="E193" s="34" t="s">
@@ -9841,7 +9582,7 @@
       <c r="C194" s="34" t="s">
         <v>848</v>
       </c>
-      <c r="D194" s="44" t="s">
+      <c r="D194" s="43" t="s">
         <v>849</v>
       </c>
       <c r="E194" s="34" t="s">
@@ -9859,7 +9600,7 @@
       <c r="C195" s="34" t="s">
         <v>358</v>
       </c>
-      <c r="D195" s="44" t="s">
+      <c r="D195" s="43" t="s">
         <v>359</v>
       </c>
       <c r="E195" s="34" t="s">
@@ -9879,7 +9620,7 @@
       <c r="C196" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D196" s="43" t="s">
+      <c r="D196" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E196" s="2" t="s">
@@ -9902,7 +9643,7 @@
       <c r="C197" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="D197" s="43" t="s">
+      <c r="D197" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E197" s="2" t="s">
@@ -9925,7 +9666,7 @@
       <c r="C198" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="D198" s="43" t="s">
+      <c r="D198" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E198" s="2" t="s">
@@ -9948,7 +9689,7 @@
       <c r="C199" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="D199" s="43" t="s">
+      <c r="D199" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E199" s="2" t="s">
@@ -9971,7 +9712,7 @@
       <c r="C200" s="4" t="s">
         <v>405</v>
       </c>
-      <c r="D200" s="43" t="s">
+      <c r="D200" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E200" s="2" t="s">
@@ -9991,7 +9732,7 @@
       <c r="C201" s="4" t="s">
         <v>444</v>
       </c>
-      <c r="D201" s="43" t="s">
+      <c r="D201" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E201" s="2" t="s">
@@ -10002,14 +9743,16 @@
       </c>
     </row>
     <row r="202" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A202" s="28"/>
+      <c r="A202" s="28" t="s">
+        <v>1565</v>
+      </c>
       <c r="B202" s="28" t="s">
         <v>474</v>
       </c>
       <c r="C202" s="28" t="s">
         <v>475</v>
       </c>
-      <c r="D202" s="43" t="s">
+      <c r="D202" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E202" s="30" t="s">
@@ -10029,7 +9772,7 @@
       <c r="C203" s="4" t="s">
         <v>515</v>
       </c>
-      <c r="D203" s="43" t="s">
+      <c r="D203" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E203" s="2" t="s">
@@ -10049,7 +9792,7 @@
       <c r="C204" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D204" s="43" t="s">
+      <c r="D204" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E204" s="5" t="s">
@@ -10073,7 +9816,7 @@
       <c r="C205" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="D205" s="43" t="s">
+      <c r="D205" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E205" s="5" t="s">
@@ -10088,14 +9831,16 @@
       <c r="P205" s="3"/>
     </row>
     <row r="206" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A206" s="28"/>
+      <c r="A206" s="28" t="s">
+        <v>1566</v>
+      </c>
       <c r="B206" s="28" t="s">
         <v>151</v>
       </c>
       <c r="C206" s="28" t="s">
         <v>152</v>
       </c>
-      <c r="D206" s="43" t="s">
+      <c r="D206" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E206" s="29" t="s">
@@ -10117,7 +9862,7 @@
       <c r="C207" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="D207" s="43" t="s">
+      <c r="D207" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E207" s="5" t="s">
@@ -10141,7 +9886,7 @@
       <c r="C208" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="D208" s="43" t="s">
+      <c r="D208" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E208" s="5" t="s">
@@ -10162,7 +9907,7 @@
       <c r="C209" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="D209" s="43" t="s">
+      <c r="D209" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E209" s="5" t="s">
@@ -10174,7 +9919,6 @@
       <c r="G209" t="s">
         <v>1554</v>
       </c>
-      <c r="I209" s="49"/>
       <c r="N209" s="7"/>
       <c r="O209" s="2"/>
     </row>
@@ -10188,7 +9932,7 @@
       <c r="C210" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="D210" s="43" t="s">
+      <c r="D210" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E210" s="5" t="s">
@@ -10212,7 +9956,7 @@
       <c r="C211" s="4" t="s">
         <v>328</v>
       </c>
-      <c r="D211" s="43" t="s">
+      <c r="D211" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E211" s="5" t="s">
@@ -10236,7 +9980,7 @@
       <c r="C212" s="34" t="s">
         <v>334</v>
       </c>
-      <c r="D212" s="43" t="s">
+      <c r="D212" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E212" s="5" t="s">
@@ -10257,7 +10001,7 @@
       <c r="C213" s="4" t="s">
         <v>336</v>
       </c>
-      <c r="D213" s="43" t="s">
+      <c r="D213" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E213" s="5" t="s">
@@ -10278,7 +10022,7 @@
       <c r="C214" s="34" t="s">
         <v>349</v>
       </c>
-      <c r="D214" s="43" t="s">
+      <c r="D214" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E214" s="5" t="s">
@@ -10299,7 +10043,7 @@
       <c r="C215" s="4" t="s">
         <v>351</v>
       </c>
-      <c r="D215" s="43" t="s">
+      <c r="D215" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E215" s="5" t="s">
@@ -10320,7 +10064,7 @@
       <c r="C216" s="4" t="s">
         <v>402</v>
       </c>
-      <c r="D216" s="43" t="s">
+      <c r="D216" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E216" s="5" t="s">
@@ -10340,7 +10084,7 @@
       <c r="C217" s="4" t="s">
         <v>473</v>
       </c>
-      <c r="D217" s="43" t="s">
+      <c r="D217" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E217" s="5" t="s">
@@ -10364,7 +10108,7 @@
       <c r="C218" s="4" t="s">
         <v>518</v>
       </c>
-      <c r="D218" s="43" t="s">
+      <c r="D218" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E218" s="5" t="s">
@@ -10385,7 +10129,7 @@
       <c r="C219" s="34" t="s">
         <v>569</v>
       </c>
-      <c r="D219" s="43" t="s">
+      <c r="D219" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E219" s="5" t="s">
@@ -10406,7 +10150,7 @@
       <c r="C220" s="4" t="s">
         <v>571</v>
       </c>
-      <c r="D220" s="43" t="s">
+      <c r="D220" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E220" s="5" t="s">
@@ -10427,7 +10171,7 @@
       <c r="C221" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="D221" s="43" t="s">
+      <c r="D221" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E221" s="5" t="s">
@@ -10449,7 +10193,7 @@
       <c r="C222" s="4" t="s">
         <v>705</v>
       </c>
-      <c r="D222" s="43" t="s">
+      <c r="D222" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E222" s="5" t="s">
@@ -10470,7 +10214,7 @@
       <c r="C223" s="4" t="s">
         <v>730</v>
       </c>
-      <c r="D223" s="43" t="s">
+      <c r="D223" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E223" s="5" t="s">
@@ -10479,7 +10223,6 @@
       <c r="F223" t="s">
         <v>18</v>
       </c>
-      <c r="I223" s="49"/>
       <c r="N223" s="7"/>
       <c r="O223" s="5"/>
     </row>
@@ -10493,7 +10236,7 @@
       <c r="C224" s="4" t="s">
         <v>744</v>
       </c>
-      <c r="D224" s="43" t="s">
+      <c r="D224" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E224" s="5" t="s">
@@ -10502,7 +10245,6 @@
       <c r="F224" t="s">
         <v>18</v>
       </c>
-      <c r="I224" s="49"/>
       <c r="J224" s="3"/>
       <c r="N224" s="10"/>
       <c r="O224" s="11"/>
@@ -10518,7 +10260,7 @@
       <c r="C225" s="4" t="s">
         <v>747</v>
       </c>
-      <c r="D225" s="43" t="s">
+      <c r="D225" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E225" s="5" t="s">
@@ -10527,7 +10269,6 @@
       <c r="F225" t="s">
         <v>18</v>
       </c>
-      <c r="I225" s="49"/>
       <c r="N225" s="7"/>
       <c r="O225" s="5"/>
     </row>
@@ -10541,7 +10282,7 @@
       <c r="C226" s="4" t="s">
         <v>799</v>
       </c>
-      <c r="D226" s="43" t="s">
+      <c r="D226" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E226" s="5" t="s">
@@ -10550,7 +10291,6 @@
       <c r="F226" t="s">
         <v>18</v>
       </c>
-      <c r="I226" s="49"/>
     </row>
     <row r="227" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A227" s="4" t="s">
@@ -10562,7 +10302,7 @@
       <c r="C227" s="4" t="s">
         <v>814</v>
       </c>
-      <c r="D227" s="43" t="s">
+      <c r="D227" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E227" s="5" t="s">
@@ -10571,7 +10311,6 @@
       <c r="F227" t="s">
         <v>18</v>
       </c>
-      <c r="I227" s="49"/>
       <c r="J227" s="3"/>
     </row>
     <row r="228" spans="1:16" x14ac:dyDescent="0.2">
@@ -10584,7 +10323,7 @@
       <c r="C228" s="4" t="s">
         <v>845</v>
       </c>
-      <c r="D228" s="43" t="s">
+      <c r="D228" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E228" s="5" t="s">
@@ -10604,7 +10343,7 @@
       <c r="C229" s="4" t="s">
         <v>880</v>
       </c>
-      <c r="D229" s="43" t="s">
+      <c r="D229" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E229" s="5" t="s">
@@ -10626,7 +10365,7 @@
       <c r="C230" s="4" t="s">
         <v>880</v>
       </c>
-      <c r="D230" s="43" t="s">
+      <c r="D230" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E230" s="5" t="s">
@@ -10646,7 +10385,7 @@
       <c r="C231" s="34" t="s">
         <v>927</v>
       </c>
-      <c r="D231" s="43" t="s">
+      <c r="D231" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E231" s="5" t="s">
@@ -10667,7 +10406,7 @@
       <c r="C232" s="4" t="s">
         <v>929</v>
       </c>
-      <c r="D232" s="43" t="s">
+      <c r="D232" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E232" s="5" t="s">
@@ -10688,7 +10427,7 @@
       <c r="C233" s="4" t="s">
         <v>959</v>
       </c>
-      <c r="D233" s="43" t="s">
+      <c r="D233" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E233" s="5" t="s">
@@ -10708,7 +10447,7 @@
       <c r="C234" s="4" t="s">
         <v>987</v>
       </c>
-      <c r="D234" s="43" t="s">
+      <c r="D234" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E234" s="5" t="s">
@@ -10732,7 +10471,7 @@
       <c r="C235" s="34" t="s">
         <v>1031</v>
       </c>
-      <c r="D235" s="43" t="s">
+      <c r="D235" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E235" s="5" t="s">
@@ -10753,7 +10492,7 @@
       <c r="C236" s="4" t="s">
         <v>1033</v>
       </c>
-      <c r="D236" s="43" t="s">
+      <c r="D236" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E236" s="5" t="s">
@@ -10774,7 +10513,7 @@
       <c r="C237" s="4" t="s">
         <v>1153</v>
       </c>
-      <c r="D237" s="43" t="s">
+      <c r="D237" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E237" s="5" t="s">
@@ -10796,7 +10535,7 @@
       <c r="C238" s="4" t="s">
         <v>1156</v>
       </c>
-      <c r="D238" s="43" t="s">
+      <c r="D238" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E238" s="5" t="s">
@@ -10811,14 +10550,16 @@
       <c r="P238" s="3"/>
     </row>
     <row r="239" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A239" s="28"/>
+      <c r="A239" s="28" t="s">
+        <v>1567</v>
+      </c>
       <c r="B239" s="28" t="s">
         <v>1162</v>
       </c>
       <c r="C239" s="28" t="s">
         <v>1163</v>
       </c>
-      <c r="D239" s="43" t="s">
+      <c r="D239" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E239" s="29" t="s">
@@ -10840,7 +10581,7 @@
       <c r="C240" s="4" t="s">
         <v>1166</v>
       </c>
-      <c r="D240" s="43" t="s">
+      <c r="D240" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E240" s="5" t="s">
@@ -10861,7 +10602,7 @@
       <c r="C241" s="4" t="s">
         <v>1172</v>
       </c>
-      <c r="D241" s="43" t="s">
+      <c r="D241" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E241" s="5" t="s">
@@ -10885,7 +10626,7 @@
       <c r="C242" s="4" t="s">
         <v>1300</v>
       </c>
-      <c r="D242" s="43" t="s">
+      <c r="D242" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E242" s="5" t="s">
@@ -10907,7 +10648,7 @@
       <c r="C243" s="4" t="s">
         <v>1350</v>
       </c>
-      <c r="D243" s="43" t="s">
+      <c r="D243" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E243" s="5" t="s">
@@ -10928,7 +10669,7 @@
       <c r="C244" s="4" t="s">
         <v>1357</v>
       </c>
-      <c r="D244" s="43" t="s">
+      <c r="D244" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E244" s="5" t="s">
@@ -10952,7 +10693,7 @@
       <c r="C245" s="4" t="s">
         <v>1365</v>
       </c>
-      <c r="D245" s="43" t="s">
+      <c r="D245" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E245" s="5" t="s">
@@ -10974,7 +10715,7 @@
       <c r="C246" s="4" t="s">
         <v>1368</v>
       </c>
-      <c r="D246" s="43" t="s">
+      <c r="D246" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E246" s="5" t="s">
@@ -10998,7 +10739,7 @@
       <c r="C247" s="4" t="s">
         <v>1390</v>
       </c>
-      <c r="D247" s="43" t="s">
+      <c r="D247" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E247" s="5" t="s">
@@ -11019,7 +10760,7 @@
       <c r="C248" s="4" t="s">
         <v>1396</v>
       </c>
-      <c r="D248" s="43" t="s">
+      <c r="D248" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E248" s="5" t="s">
@@ -11039,7 +10780,7 @@
       <c r="C249" s="34" t="s">
         <v>1398</v>
       </c>
-      <c r="D249" s="43" t="s">
+      <c r="D249" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E249" s="5" t="s">
@@ -11060,7 +10801,7 @@
       <c r="C250" s="4" t="s">
         <v>1402</v>
       </c>
-      <c r="D250" s="43" t="s">
+      <c r="D250" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E250" s="5" t="s">
@@ -11085,7 +10826,7 @@
       <c r="C251" s="4" t="s">
         <v>1452</v>
       </c>
-      <c r="D251" s="43" t="s">
+      <c r="D251" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E251" s="5" t="s">
@@ -11105,7 +10846,7 @@
       <c r="C252" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D252" s="43" t="s">
+      <c r="D252" s="15" t="s">
         <v>114</v>
       </c>
       <c r="E252" s="5" t="s">
@@ -11127,7 +10868,7 @@
       <c r="C253" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D253" s="43" t="s">
+      <c r="D253" s="15" t="s">
         <v>114</v>
       </c>
       <c r="E253" s="5" t="s">
@@ -11149,7 +10890,7 @@
       <c r="C254" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D254" s="43" t="s">
+      <c r="D254" s="15" t="s">
         <v>114</v>
       </c>
       <c r="E254" t="s">
@@ -11169,7 +10910,7 @@
       <c r="C255" s="4" t="s">
         <v>763</v>
       </c>
-      <c r="D255" s="43" t="s">
+      <c r="D255" s="15" t="s">
         <v>114</v>
       </c>
       <c r="E255" s="5" t="s">
@@ -11191,7 +10932,7 @@
       <c r="C256" s="4" t="s">
         <v>901</v>
       </c>
-      <c r="D256" s="43" t="s">
+      <c r="D256" s="15" t="s">
         <v>114</v>
       </c>
       <c r="E256" s="5" t="s">
@@ -11216,7 +10957,7 @@
       <c r="C257" s="4" t="s">
         <v>903</v>
       </c>
-      <c r="D257" s="43" t="s">
+      <c r="D257" s="15" t="s">
         <v>114</v>
       </c>
       <c r="E257" s="5" t="s">
@@ -11238,7 +10979,7 @@
       <c r="C258" s="34" t="s">
         <v>178</v>
       </c>
-      <c r="D258" s="43" t="s">
+      <c r="D258" s="15" t="s">
         <v>179</v>
       </c>
       <c r="E258" s="5" t="s">
@@ -11259,7 +11000,7 @@
       <c r="C259" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="D259" s="43" t="s">
+      <c r="D259" s="15" t="s">
         <v>179</v>
       </c>
       <c r="E259" s="5" t="s">
@@ -11281,7 +11022,7 @@
       <c r="C260" s="4" t="s">
         <v>310</v>
       </c>
-      <c r="D260" s="43" t="s">
+      <c r="D260" s="15" t="s">
         <v>311</v>
       </c>
       <c r="E260" s="5" t="s">
@@ -11303,7 +11044,7 @@
       <c r="C261" s="4" t="s">
         <v>758</v>
       </c>
-      <c r="D261" s="43" t="s">
+      <c r="D261" s="15" t="s">
         <v>759</v>
       </c>
       <c r="E261" s="2" t="s">
@@ -11325,7 +11066,7 @@
       <c r="C262" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="D262" s="43" t="s">
+      <c r="D262" s="15" t="s">
         <v>138</v>
       </c>
       <c r="E262" s="5" t="s">
@@ -11347,7 +11088,7 @@
       <c r="C263" s="4" t="s">
         <v>1016</v>
       </c>
-      <c r="D263" s="43" t="s">
+      <c r="D263" s="15" t="s">
         <v>138</v>
       </c>
       <c r="E263" s="5" t="s">
@@ -11369,7 +11110,7 @@
       <c r="C264" s="4" t="s">
         <v>1019</v>
       </c>
-      <c r="D264" s="43" t="s">
+      <c r="D264" s="15" t="s">
         <v>138</v>
       </c>
       <c r="E264" t="s">
@@ -11389,7 +11130,7 @@
       <c r="C265" s="34" t="s">
         <v>806</v>
       </c>
-      <c r="D265" s="44" t="s">
+      <c r="D265" s="43" t="s">
         <v>807</v>
       </c>
       <c r="E265" s="34" t="s">
@@ -11407,7 +11148,7 @@
       <c r="C266" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D266" s="43" t="s">
+      <c r="D266" s="15" t="s">
         <v>16</v>
       </c>
       <c r="E266" t="s">
@@ -11427,7 +11168,7 @@
       <c r="C267" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="D267" s="43" t="s">
+      <c r="D267" s="15" t="s">
         <v>16</v>
       </c>
       <c r="E267" s="5" t="s">
@@ -11449,7 +11190,7 @@
       <c r="C268" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="D268" s="43" t="s">
+      <c r="D268" s="15" t="s">
         <v>286</v>
       </c>
       <c r="E268" s="16" t="s">
@@ -11469,7 +11210,7 @@
       <c r="C269" s="4" t="s">
         <v>1140</v>
       </c>
-      <c r="D269" s="43" t="s">
+      <c r="D269" s="15" t="s">
         <v>286</v>
       </c>
       <c r="E269" s="16" t="s">
@@ -11489,7 +11230,7 @@
       <c r="C270" s="34" t="s">
         <v>1311</v>
       </c>
-      <c r="D270" s="45" t="s">
+      <c r="D270" s="22" t="s">
         <v>286</v>
       </c>
       <c r="E270" s="34" t="s">
@@ -11509,7 +11250,7 @@
       <c r="C271" s="34" t="s">
         <v>1314</v>
       </c>
-      <c r="D271" s="44" t="s">
+      <c r="D271" s="43" t="s">
         <v>1315</v>
       </c>
       <c r="E271" s="34" t="s">
@@ -11529,7 +11270,7 @@
       <c r="C272" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="D272" s="44" t="s">
+      <c r="D272" s="43" t="s">
         <v>77</v>
       </c>
       <c r="E272" s="34" t="s">
@@ -11549,7 +11290,7 @@
       <c r="C273" s="33" t="s">
         <v>413</v>
       </c>
-      <c r="D273" s="44" t="s">
+      <c r="D273" s="43" t="s">
         <v>77</v>
       </c>
       <c r="E273" s="34" t="s">
@@ -11569,7 +11310,7 @@
       <c r="C274" s="34" t="s">
         <v>415</v>
       </c>
-      <c r="D274" s="44" t="s">
+      <c r="D274" s="43" t="s">
         <v>77</v>
       </c>
       <c r="E274" s="34" t="s">
@@ -11589,7 +11330,7 @@
       <c r="C275" s="33" t="s">
         <v>1410</v>
       </c>
-      <c r="D275" s="44" t="s">
+      <c r="D275" s="43" t="s">
         <v>1411</v>
       </c>
       <c r="E275" s="34" t="s">
@@ -11609,7 +11350,7 @@
       <c r="C276" s="33" t="s">
         <v>1230</v>
       </c>
-      <c r="D276" s="44" t="s">
+      <c r="D276" s="43" t="s">
         <v>1231</v>
       </c>
       <c r="E276" s="34" t="s">
@@ -11629,7 +11370,7 @@
       <c r="C277" s="33" t="s">
         <v>582</v>
       </c>
-      <c r="D277" s="44" t="s">
+      <c r="D277" s="43" t="s">
         <v>583</v>
       </c>
       <c r="E277" s="34" t="s">
@@ -11649,7 +11390,7 @@
       <c r="C278" s="33" t="s">
         <v>664</v>
       </c>
-      <c r="D278" s="44" t="s">
+      <c r="D278" s="43" t="s">
         <v>665</v>
       </c>
       <c r="E278" s="34" t="s">
@@ -11669,7 +11410,7 @@
       <c r="C279" s="33" t="s">
         <v>485</v>
       </c>
-      <c r="D279" s="44" t="s">
+      <c r="D279" s="43" t="s">
         <v>486</v>
       </c>
       <c r="E279" s="34" t="s">
@@ -11689,7 +11430,7 @@
       <c r="C280" s="35" t="s">
         <v>592</v>
       </c>
-      <c r="D280" s="44" t="s">
+      <c r="D280" s="43" t="s">
         <v>486</v>
       </c>
       <c r="E280" s="36" t="s">
@@ -11709,7 +11450,7 @@
       <c r="C281" s="33" t="s">
         <v>1101</v>
       </c>
-      <c r="D281" s="44" t="s">
+      <c r="D281" s="43" t="s">
         <v>486</v>
       </c>
       <c r="E281" s="34" t="s">
@@ -11729,7 +11470,7 @@
       <c r="C282" s="33" t="s">
         <v>678</v>
       </c>
-      <c r="D282" s="44" t="s">
+      <c r="D282" s="43" t="s">
         <v>679</v>
       </c>
       <c r="E282" s="34" t="s">
@@ -11749,7 +11490,7 @@
       <c r="C283" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="D283" s="43" t="s">
+      <c r="D283" s="15" t="s">
         <v>167</v>
       </c>
       <c r="E283" t="s">
@@ -11769,7 +11510,7 @@
       <c r="C284" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="D284" s="43" t="s">
+      <c r="D284" s="15" t="s">
         <v>167</v>
       </c>
       <c r="E284" t="s">
@@ -11789,7 +11530,7 @@
       <c r="C285" s="4" t="s">
         <v>1047</v>
       </c>
-      <c r="D285" s="46" t="s">
+      <c r="D285" s="44" t="s">
         <v>1048</v>
       </c>
       <c r="E285" t="s">
@@ -11809,7 +11550,7 @@
       <c r="C286" s="33" t="s">
         <v>641</v>
       </c>
-      <c r="D286" s="44" t="s">
+      <c r="D286" s="43" t="s">
         <v>642</v>
       </c>
       <c r="E286" s="34" t="s">
@@ -11829,7 +11570,7 @@
       <c r="C287" s="4" t="s">
         <v>1116</v>
       </c>
-      <c r="D287" s="43" t="s">
+      <c r="D287" s="15" t="s">
         <v>642</v>
       </c>
       <c r="E287" t="s">
@@ -11849,7 +11590,7 @@
       <c r="C288" s="4" t="s">
         <v>1235</v>
       </c>
-      <c r="D288" s="43" t="s">
+      <c r="D288" s="15" t="s">
         <v>1236</v>
       </c>
       <c r="E288" t="s">
@@ -11869,7 +11610,7 @@
       <c r="C289" s="4" t="s">
         <v>587</v>
       </c>
-      <c r="D289" s="43" t="s">
+      <c r="D289" s="15" t="s">
         <v>588</v>
       </c>
       <c r="E289" t="s">
@@ -11889,7 +11630,7 @@
       <c r="C290" s="4" t="s">
         <v>500</v>
       </c>
-      <c r="D290" s="43" t="s">
+      <c r="D290" s="15" t="s">
         <v>501</v>
       </c>
       <c r="E290" t="s">
@@ -11909,7 +11650,7 @@
       <c r="C291" s="34" t="s">
         <v>305</v>
       </c>
-      <c r="D291" s="44" t="s">
+      <c r="D291" s="43" t="s">
         <v>306</v>
       </c>
       <c r="E291" s="34" t="s">
@@ -11929,7 +11670,7 @@
       <c r="C292" s="33" t="s">
         <v>622</v>
       </c>
-      <c r="D292" s="44" t="s">
+      <c r="D292" s="43" t="s">
         <v>306</v>
       </c>
       <c r="E292" s="34" t="s">
@@ -11949,7 +11690,7 @@
       <c r="C293" s="33" t="s">
         <v>490</v>
       </c>
-      <c r="D293" s="44" t="s">
+      <c r="D293" s="43" t="s">
         <v>491</v>
       </c>
       <c r="E293" s="34" t="s">
@@ -11969,7 +11710,7 @@
       <c r="C294" s="33" t="s">
         <v>595</v>
       </c>
-      <c r="D294" s="44" t="s">
+      <c r="D294" s="43" t="s">
         <v>596</v>
       </c>
       <c r="E294" s="34" t="s">
@@ -11989,7 +11730,7 @@
       <c r="C295" s="33" t="s">
         <v>1385</v>
       </c>
-      <c r="D295" s="44" t="s">
+      <c r="D295" s="43" t="s">
         <v>1386</v>
       </c>
       <c r="E295" s="34" t="s">
@@ -12009,7 +11750,7 @@
       <c r="C296" s="33" t="s">
         <v>1052</v>
       </c>
-      <c r="D296" s="44" t="s">
+      <c r="D296" s="43" t="s">
         <v>1053</v>
       </c>
       <c r="E296" s="34" t="s">
@@ -12029,7 +11770,7 @@
       <c r="C297" s="33" t="s">
         <v>468</v>
       </c>
-      <c r="D297" s="44" t="s">
+      <c r="D297" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E297" s="34" t="s">
@@ -12049,7 +11790,7 @@
       <c r="C298" s="33" t="s">
         <v>508</v>
       </c>
-      <c r="D298" s="44" t="s">
+      <c r="D298" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E298" s="34" t="s">
@@ -12069,7 +11810,7 @@
       <c r="C299" s="33" t="s">
         <v>831</v>
       </c>
-      <c r="D299" s="44" t="s">
+      <c r="D299" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E299" s="34" t="s">
@@ -12089,7 +11830,7 @@
       <c r="C300" s="33" t="s">
         <v>996</v>
       </c>
-      <c r="D300" s="44" t="s">
+      <c r="D300" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E300" s="34" t="s">
@@ -12109,7 +11850,7 @@
       <c r="C301" s="33" t="s">
         <v>1041</v>
       </c>
-      <c r="D301" s="44" t="s">
+      <c r="D301" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E301" s="34" t="s">
@@ -12129,7 +11870,7 @@
       <c r="C302" s="33" t="s">
         <v>1104</v>
       </c>
-      <c r="D302" s="44" t="s">
+      <c r="D302" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E302" s="34" t="s">
@@ -12149,7 +11890,7 @@
       <c r="C303" s="33" t="s">
         <v>1130</v>
       </c>
-      <c r="D303" s="44" t="s">
+      <c r="D303" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E303" s="34" t="s">
@@ -12169,7 +11910,7 @@
       <c r="C304" s="33" t="s">
         <v>1137</v>
       </c>
-      <c r="D304" s="44" t="s">
+      <c r="D304" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E304" s="34" t="s">
@@ -12189,7 +11930,7 @@
       <c r="C305" s="33" t="s">
         <v>1441</v>
       </c>
-      <c r="D305" s="44" t="s">
+      <c r="D305" s="43" t="s">
         <v>469</v>
       </c>
       <c r="E305" s="34" t="s">
@@ -12209,7 +11950,7 @@
       <c r="C306" s="4" t="s">
         <v>674</v>
       </c>
-      <c r="D306" s="47" t="s">
+      <c r="D306" s="45" t="s">
         <v>675</v>
       </c>
       <c r="E306" s="4" t="s">
@@ -12229,7 +11970,7 @@
       <c r="C307" s="4" t="s">
         <v>669</v>
       </c>
-      <c r="D307" s="47" t="s">
+      <c r="D307" s="45" t="s">
         <v>670</v>
       </c>
       <c r="E307" s="4" t="s">
@@ -12252,7 +11993,7 @@
       <c r="C308" s="4" t="s">
         <v>1285</v>
       </c>
-      <c r="D308" s="47" t="s">
+      <c r="D308" s="45" t="s">
         <v>1286</v>
       </c>
       <c r="E308" s="4" t="s">
@@ -12272,7 +12013,7 @@
       <c r="C309" s="4" t="s">
         <v>511</v>
       </c>
-      <c r="D309" s="47" t="s">
+      <c r="D309" s="45" t="s">
         <v>512</v>
       </c>
       <c r="E309" s="4" t="s">
@@ -12292,7 +12033,7 @@
       <c r="C310" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D310" s="47" t="s">
+      <c r="D310" s="45" t="s">
         <v>41</v>
       </c>
       <c r="E310" s="4" t="s">
@@ -12312,7 +12053,7 @@
       <c r="C311" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="D311" s="47" t="s">
+      <c r="D311" s="45" t="s">
         <v>282</v>
       </c>
       <c r="E311" s="4" t="s">
@@ -12332,7 +12073,7 @@
       <c r="C312" s="4" t="s">
         <v>1243</v>
       </c>
-      <c r="D312" s="47" t="s">
+      <c r="D312" s="45" t="s">
         <v>1244</v>
       </c>
       <c r="E312" s="4" t="s">
@@ -12352,7 +12093,7 @@
       <c r="C313" s="4" t="s">
         <v>1437</v>
       </c>
-      <c r="D313" s="47" t="s">
+      <c r="D313" s="45" t="s">
         <v>1438</v>
       </c>
       <c r="E313" s="4" t="s">
@@ -12372,7 +12113,7 @@
       <c r="C314" s="4" t="s">
         <v>1036</v>
       </c>
-      <c r="D314" s="47" t="s">
+      <c r="D314" s="45" t="s">
         <v>1037</v>
       </c>
       <c r="E314" s="4" t="s">
@@ -12392,7 +12133,7 @@
       <c r="C315" s="4" t="s">
         <v>1203</v>
       </c>
-      <c r="D315" s="47" t="s">
+      <c r="D315" s="45" t="s">
         <v>1204</v>
       </c>
       <c r="E315" s="4" t="s">
@@ -12412,7 +12153,7 @@
       <c r="C316" s="4" t="s">
         <v>817</v>
       </c>
-      <c r="D316" s="47" t="s">
+      <c r="D316" s="45" t="s">
         <v>818</v>
       </c>
       <c r="E316" s="4" t="s">
@@ -12432,7 +12173,7 @@
       <c r="C317" s="4" t="s">
         <v>1381</v>
       </c>
-      <c r="D317" s="47" t="s">
+      <c r="D317" s="45" t="s">
         <v>1382</v>
       </c>
       <c r="E317" s="4" t="s">
@@ -12452,7 +12193,7 @@
       <c r="C318" s="4" t="s">
         <v>897</v>
       </c>
-      <c r="D318" s="47" t="s">
+      <c r="D318" s="45" t="s">
         <v>898</v>
       </c>
       <c r="E318" s="4" t="s">
@@ -12472,7 +12213,7 @@
       <c r="C319" s="4" t="s">
         <v>633</v>
       </c>
-      <c r="D319" s="47" t="s">
+      <c r="D319" s="45" t="s">
         <v>634</v>
       </c>
       <c r="E319" s="4" t="s">
@@ -12492,7 +12233,7 @@
       <c r="C320" s="4" t="s">
         <v>531</v>
       </c>
-      <c r="D320" s="47" t="s">
+      <c r="D320" s="45" t="s">
         <v>532</v>
       </c>
       <c r="E320" s="4" t="s">
@@ -12512,7 +12253,7 @@
       <c r="C321" s="4" t="s">
         <v>637</v>
       </c>
-      <c r="D321" s="47" t="s">
+      <c r="D321" s="45" t="s">
         <v>638</v>
       </c>
       <c r="E321" s="4" t="s">
@@ -12532,7 +12273,7 @@
       <c r="C322" s="4" t="s">
         <v>1071</v>
       </c>
-      <c r="D322" s="47" t="s">
+      <c r="D322" s="45" t="s">
         <v>1072</v>
       </c>
       <c r="E322" s="4" t="s">
@@ -12552,7 +12293,7 @@
       <c r="C323" s="4" t="s">
         <v>1254</v>
       </c>
-      <c r="D323" s="47" t="s">
+      <c r="D323" s="45" t="s">
         <v>1255</v>
       </c>
       <c r="E323" s="4" t="s">
@@ -12572,7 +12313,7 @@
       <c r="C324" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="D324" s="47" t="s">
+      <c r="D324" s="45" t="s">
         <v>236</v>
       </c>
       <c r="E324" s="4" t="s">
@@ -12592,7 +12333,7 @@
       <c r="C325" s="4" t="s">
         <v>535</v>
       </c>
-      <c r="D325" s="47" t="s">
+      <c r="D325" s="45" t="s">
         <v>536</v>
       </c>
       <c r="E325" s="4" t="s">
@@ -12612,7 +12353,7 @@
       <c r="C326" s="4" t="s">
         <v>1146</v>
       </c>
-      <c r="D326" s="47" t="s">
+      <c r="D326" s="45" t="s">
         <v>1147</v>
       </c>
       <c r="E326" s="4" t="s">
@@ -12632,7 +12373,7 @@
       <c r="C327" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D327" s="47" t="s">
+      <c r="D327" s="45" t="s">
         <v>46</v>
       </c>
       <c r="E327" s="4" t="s">
@@ -12652,7 +12393,7 @@
       <c r="C328" s="4" t="s">
         <v>1226</v>
       </c>
-      <c r="D328" s="47" t="s">
+      <c r="D328" s="45" t="s">
         <v>1227</v>
       </c>
       <c r="E328" s="4" t="s">
@@ -12672,7 +12413,7 @@
       <c r="C329" s="4" t="s">
         <v>1133</v>
       </c>
-      <c r="D329" s="47" t="s">
+      <c r="D329" s="45" t="s">
         <v>1134</v>
       </c>
       <c r="E329" s="4" t="s">
@@ -12692,7 +12433,7 @@
       <c r="C330" s="4" t="s">
         <v>1303</v>
       </c>
-      <c r="D330" s="47" t="s">
+      <c r="D330" s="45" t="s">
         <v>1304</v>
       </c>
       <c r="E330" s="4" t="s">
@@ -12712,7 +12453,7 @@
       <c r="C331" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D331" s="47" t="s">
+      <c r="D331" s="45" t="s">
         <v>150</v>
       </c>
       <c r="E331" s="4" t="s">
@@ -12732,7 +12473,7 @@
       <c r="C332" s="4" t="s">
         <v>1195</v>
       </c>
-      <c r="D332" s="47" t="s">
+      <c r="D332" s="45" t="s">
         <v>1196</v>
       </c>
       <c r="E332" s="4" t="s">
@@ -12752,7 +12493,7 @@
       <c r="C333" s="4" t="s">
         <v>1338</v>
       </c>
-      <c r="D333" s="47" t="s">
+      <c r="D333" s="45" t="s">
         <v>1339</v>
       </c>
       <c r="E333" s="4" t="s">
@@ -12772,7 +12513,7 @@
       <c r="C334" s="4" t="s">
         <v>539</v>
       </c>
-      <c r="D334" s="47" t="s">
+      <c r="D334" s="45" t="s">
         <v>540</v>
       </c>
       <c r="E334" s="4" t="s">
@@ -12792,7 +12533,7 @@
       <c r="C335" s="4" t="s">
         <v>787</v>
       </c>
-      <c r="D335" s="47" t="s">
+      <c r="D335" s="45" t="s">
         <v>788</v>
       </c>
       <c r="E335" s="4" t="s">
@@ -12812,7 +12553,7 @@
       <c r="C336" s="4" t="s">
         <v>783</v>
       </c>
-      <c r="D336" s="47" t="s">
+      <c r="D336" s="45" t="s">
         <v>784</v>
       </c>
       <c r="E336" s="4" t="s">
@@ -12832,7 +12573,7 @@
       <c r="C337" s="4" t="s">
         <v>1085</v>
       </c>
-      <c r="D337" s="47" t="s">
+      <c r="D337" s="45" t="s">
         <v>1086</v>
       </c>
       <c r="E337" s="4" t="s">
@@ -12852,7 +12593,7 @@
       <c r="C338" s="4" t="s">
         <v>1433</v>
       </c>
-      <c r="D338" s="47" t="s">
+      <c r="D338" s="45" t="s">
         <v>1434</v>
       </c>
       <c r="E338" s="4" t="s">
@@ -12872,7 +12613,7 @@
       <c r="C339" s="4" t="s">
         <v>1281</v>
       </c>
-      <c r="D339" s="47" t="s">
+      <c r="D339" s="45" t="s">
         <v>1282</v>
       </c>
       <c r="E339" s="4" t="s">
@@ -12892,7 +12633,7 @@
       <c r="C340" s="4" t="s">
         <v>543</v>
       </c>
-      <c r="D340" s="47" t="s">
+      <c r="D340" s="45" t="s">
         <v>544</v>
       </c>
       <c r="E340" s="4" t="s">
@@ -12912,7 +12653,7 @@
       <c r="C341" s="4" t="s">
         <v>1292</v>
       </c>
-      <c r="D341" s="47" t="s">
+      <c r="D341" s="45" t="s">
         <v>1293</v>
       </c>
       <c r="E341" s="4" t="s">
@@ -12932,7 +12673,7 @@
       <c r="C342" s="4" t="s">
         <v>937</v>
       </c>
-      <c r="D342" s="47" t="s">
+      <c r="D342" s="45" t="s">
         <v>938</v>
       </c>
       <c r="E342" s="4" t="s">
@@ -12952,7 +12693,7 @@
       <c r="C343" s="4" t="s">
         <v>452</v>
       </c>
-      <c r="D343" s="47" t="s">
+      <c r="D343" s="45" t="s">
         <v>453</v>
       </c>
       <c r="E343" s="4" t="s">
@@ -12972,7 +12713,7 @@
       <c r="C344" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="D344" s="47" t="s">
+      <c r="D344" s="45" t="s">
         <v>343</v>
       </c>
       <c r="E344" s="4" t="s">
@@ -12992,7 +12733,7 @@
       <c r="C345" s="4" t="s">
         <v>354</v>
       </c>
-      <c r="D345" s="47" t="s">
+      <c r="D345" s="45" t="s">
         <v>355</v>
       </c>
       <c r="E345" s="4" t="s">
@@ -13012,7 +12753,7 @@
       <c r="C346" s="4" t="s">
         <v>906</v>
       </c>
-      <c r="D346" s="47" t="s">
+      <c r="D346" s="45" t="s">
         <v>907</v>
       </c>
       <c r="E346" s="4" t="s">
@@ -13032,7 +12773,7 @@
       <c r="C347" s="4" t="s">
         <v>968</v>
       </c>
-      <c r="D347" s="47" t="s">
+      <c r="D347" s="45" t="s">
         <v>969</v>
       </c>
       <c r="E347" s="4" t="s">
@@ -13052,7 +12793,7 @@
       <c r="C348" s="4" t="s">
         <v>1199</v>
       </c>
-      <c r="D348" s="47" t="s">
+      <c r="D348" s="45" t="s">
         <v>1200</v>
       </c>
       <c r="E348" s="4" t="s">
@@ -13072,7 +12813,7 @@
       <c r="C349" s="4" t="s">
         <v>1428</v>
       </c>
-      <c r="D349" s="47" t="s">
+      <c r="D349" s="45" t="s">
         <v>1429</v>
       </c>
       <c r="E349" s="4" t="s">
@@ -13092,7 +12833,7 @@
       <c r="C350" s="4" t="s">
         <v>1449</v>
       </c>
-      <c r="D350" s="47" t="s">
+      <c r="D350" s="45" t="s">
         <v>1429</v>
       </c>
       <c r="E350" s="4" t="s">
@@ -13112,7 +12853,7 @@
       <c r="C351" s="4" t="s">
         <v>547</v>
       </c>
-      <c r="D351" s="47" t="s">
+      <c r="D351" s="45" t="s">
         <v>548</v>
       </c>
       <c r="E351" s="4" t="s">
@@ -13132,7 +12873,7 @@
       <c r="C352" s="4" t="s">
         <v>1247</v>
       </c>
-      <c r="D352" s="47" t="s">
+      <c r="D352" s="45" t="s">
         <v>1248</v>
       </c>
       <c r="E352" s="4" t="s">
@@ -13152,7 +12893,7 @@
       <c r="C353" s="4" t="s">
         <v>1175</v>
       </c>
-      <c r="D353" s="47" t="s">
+      <c r="D353" s="45" t="s">
         <v>1176</v>
       </c>
       <c r="E353" s="4" t="s">
@@ -13172,7 +12913,7 @@
       <c r="C354" s="4" t="s">
         <v>1374</v>
       </c>
-      <c r="D354" s="47" t="s">
+      <c r="D354" s="45" t="s">
         <v>1375</v>
       </c>
       <c r="E354" s="4" t="s">
@@ -13192,7 +12933,7 @@
       <c r="C355" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="D355" s="47" t="s">
+      <c r="D355" s="45" t="s">
         <v>258</v>
       </c>
       <c r="E355" s="4" t="s">
@@ -13212,7 +12953,7 @@
       <c r="C356" s="4" t="s">
         <v>1458</v>
       </c>
-      <c r="D356" s="47" t="s">
+      <c r="D356" s="45" t="s">
         <v>1459</v>
       </c>
       <c r="E356" s="4" t="s">
@@ -13232,7 +12973,7 @@
       <c r="C357" s="4" t="s">
         <v>368</v>
       </c>
-      <c r="D357" s="47" t="s">
+      <c r="D357" s="45" t="s">
         <v>369</v>
       </c>
       <c r="E357" s="4" t="s">
@@ -13252,7 +12993,7 @@
       <c r="C358" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="D358" s="47" t="s">
+      <c r="D358" s="45" t="s">
         <v>373</v>
       </c>
       <c r="E358" s="4" t="s">
@@ -13275,7 +13016,7 @@
       <c r="C359" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="D359" s="47" t="s">
+      <c r="D359" s="45" t="s">
         <v>378</v>
       </c>
       <c r="E359" s="4" t="s">
@@ -13298,7 +13039,7 @@
       <c r="C360" s="4" t="s">
         <v>1213</v>
       </c>
-      <c r="D360" s="47" t="s">
+      <c r="D360" s="45" t="s">
         <v>1214</v>
       </c>
       <c r="E360" s="4" t="s">
@@ -13319,7 +13060,7 @@
       <c r="C361" s="4" t="s">
         <v>629</v>
       </c>
-      <c r="D361" s="47" t="s">
+      <c r="D361" s="45" t="s">
         <v>630</v>
       </c>
       <c r="E361" s="4" t="s">
@@ -13339,7 +13080,7 @@
       <c r="C362" s="4" t="s">
         <v>802</v>
       </c>
-      <c r="D362" s="47" t="s">
+      <c r="D362" s="45" t="s">
         <v>803</v>
       </c>
       <c r="E362" s="4" t="s">
@@ -13359,7 +13100,7 @@
       <c r="C363" t="s">
         <v>685</v>
       </c>
-      <c r="D363" s="43" t="s">
+      <c r="D363" s="15" t="s">
         <v>686</v>
       </c>
       <c r="E363" t="s">
@@ -13367,14 +13108,16 @@
       </c>
     </row>
     <row r="364" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A364" s="28"/>
+      <c r="A364" t="s">
+        <v>683</v>
+      </c>
       <c r="B364" s="28" t="s">
         <v>684</v>
       </c>
       <c r="C364" s="28" t="s">
         <v>687</v>
       </c>
-      <c r="D364" s="43" t="s">
+      <c r="D364" s="15" t="s">
         <v>686</v>
       </c>
       <c r="E364" t="s">
@@ -13399,7 +13142,7 @@
       <c r="C365" t="s">
         <v>72</v>
       </c>
-      <c r="D365" s="43" t="s">
+      <c r="D365" s="15" t="s">
         <v>73</v>
       </c>
       <c r="E365" t="s">
@@ -13416,7 +13159,7 @@
       <c r="C366" t="s">
         <v>8</v>
       </c>
-      <c r="D366" s="43" t="s">
+      <c r="D366" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E366" t="s">
@@ -13433,7 +13176,7 @@
       <c r="C367" t="s">
         <v>1307</v>
       </c>
-      <c r="D367" s="43" t="s">
+      <c r="D367" s="15" t="s">
         <v>1308</v>
       </c>
       <c r="E367" t="s">
@@ -13450,7 +13193,7 @@
       <c r="C368" s="4" t="s">
         <v>478</v>
       </c>
-      <c r="D368" s="43" t="s">
+      <c r="D368" s="15" t="s">
         <v>479</v>
       </c>
       <c r="E368" s="2" t="s">
@@ -13474,7 +13217,7 @@
       <c r="C369" t="s">
         <v>1353</v>
       </c>
-      <c r="D369" s="43" t="s">
+      <c r="D369" s="15" t="s">
         <v>1354</v>
       </c>
       <c r="E369" t="s">
@@ -13498,7 +13241,7 @@
       <c r="C370" s="4" t="s">
         <v>1422</v>
       </c>
-      <c r="D370" s="43" t="s">
+      <c r="D370" s="15" t="s">
         <v>1423</v>
       </c>
       <c r="E370" t="s">
@@ -13522,7 +13265,7 @@
       <c r="C371" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D371" s="43" t="s">
+      <c r="D371" s="15" t="s">
         <v>156</v>
       </c>
       <c r="E371" t="s">
@@ -13546,7 +13289,7 @@
       <c r="C372" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D372" s="43" t="s">
+      <c r="D372" s="15" t="s">
         <v>159</v>
       </c>
       <c r="E372" t="s">
@@ -13570,7 +13313,7 @@
       <c r="C373" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D373" s="43" t="s">
+      <c r="D373" s="15" t="s">
         <v>162</v>
       </c>
       <c r="E373" t="s">
@@ -13579,8 +13322,6 @@
       <c r="F373" t="s">
         <v>157</v>
       </c>
-      <c r="J373" s="49"/>
-      <c r="K373" s="49"/>
       <c r="N373" s="8"/>
       <c r="O373" s="9"/>
       <c r="P373" s="1"/>
@@ -13596,7 +13337,7 @@
       <c r="C374" s="4" t="s">
         <v>478</v>
       </c>
-      <c r="D374" s="43" t="s">
+      <c r="D374" s="15" t="s">
         <v>481</v>
       </c>
       <c r="E374" t="s">
@@ -13605,8 +13346,6 @@
       <c r="F374" t="s">
         <v>157</v>
       </c>
-      <c r="J374" s="49"/>
-      <c r="K374" s="49"/>
       <c r="N374" s="10"/>
       <c r="O374" s="11"/>
       <c r="P374" s="3"/>
@@ -13621,7 +13360,7 @@
       <c r="C375" s="4" t="s">
         <v>1182</v>
       </c>
-      <c r="D375" s="43" t="s">
+      <c r="D375" s="15" t="s">
         <v>1183</v>
       </c>
       <c r="E375" s="4" t="s">
@@ -13630,8 +13369,6 @@
       <c r="F375" t="s">
         <v>18</v>
       </c>
-      <c r="J375" s="49"/>
-      <c r="K375" s="49"/>
     </row>
     <row r="376" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A376" t="s">
@@ -13643,14 +13380,12 @@
       <c r="C376" t="s">
         <v>1182</v>
       </c>
-      <c r="D376" s="43" t="s">
+      <c r="D376" s="15" t="s">
         <v>1183</v>
       </c>
       <c r="E376" t="s">
         <v>1182</v>
       </c>
-      <c r="J376" s="49"/>
-      <c r="K376" s="49"/>
     </row>
     <row r="377" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A377" s="4" t="s">
@@ -13662,7 +13397,7 @@
       <c r="C377" s="4" t="s">
         <v>1186</v>
       </c>
-      <c r="D377" s="43" t="s">
+      <c r="D377" s="15" t="s">
         <v>1183</v>
       </c>
       <c r="E377" s="4" t="s">
@@ -13671,8 +13406,6 @@
       <c r="F377" t="s">
         <v>18</v>
       </c>
-      <c r="J377" s="49"/>
-      <c r="K377" s="49"/>
     </row>
     <row r="378" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A378" s="4" t="s">
@@ -13684,7 +13417,7 @@
       <c r="C378" s="4" t="s">
         <v>1189</v>
       </c>
-      <c r="D378" s="43" t="s">
+      <c r="D378" s="15" t="s">
         <v>1183</v>
       </c>
       <c r="E378" s="4" t="s">
@@ -13693,8 +13426,6 @@
       <c r="F378" t="s">
         <v>18</v>
       </c>
-      <c r="J378" s="49"/>
-      <c r="K378" s="49"/>
     </row>
     <row r="379" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A379" s="4" t="s">
@@ -13706,7 +13437,7 @@
       <c r="C379" s="4" t="s">
         <v>1192</v>
       </c>
-      <c r="D379" s="43" t="s">
+      <c r="D379" s="15" t="s">
         <v>1183</v>
       </c>
       <c r="E379" s="4" t="s">
@@ -13715,8 +13446,6 @@
       <c r="F379" t="s">
         <v>18</v>
       </c>
-      <c r="J379" s="49"/>
-      <c r="K379" s="49"/>
     </row>
     <row r="380" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A380" s="4" t="s">
@@ -13728,7 +13457,7 @@
       <c r="C380" s="4" t="s">
         <v>1210</v>
       </c>
-      <c r="D380" s="43" t="s">
+      <c r="D380" s="15" t="s">
         <v>1183</v>
       </c>
       <c r="E380" s="4" t="s">
@@ -13737,8 +13466,6 @@
       <c r="F380" t="s">
         <v>18</v>
       </c>
-      <c r="J380" s="49"/>
-      <c r="K380" s="49"/>
     </row>
     <row r="381" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A381" t="s">
@@ -13750,14 +13477,12 @@
       <c r="C381" t="s">
         <v>1472</v>
       </c>
-      <c r="D381" s="43" t="s">
+      <c r="D381" s="15" t="s">
         <v>1473</v>
       </c>
       <c r="E381" t="s">
         <v>1472</v>
       </c>
-      <c r="J381" s="49"/>
-      <c r="K381" s="49"/>
     </row>
     <row r="382" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A382" t="s">
@@ -13769,14 +13494,12 @@
       <c r="C382" t="s">
         <v>887</v>
       </c>
-      <c r="D382" s="43" t="s">
+      <c r="D382" s="15" t="s">
         <v>888</v>
       </c>
       <c r="E382" t="s">
         <v>887</v>
       </c>
-      <c r="J382" s="49"/>
-      <c r="K382" s="49"/>
     </row>
     <row r="383" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A383" t="s">
@@ -13788,14 +13511,12 @@
       <c r="C383" t="s">
         <v>776</v>
       </c>
-      <c r="D383" s="43" t="s">
+      <c r="D383" s="15" t="s">
         <v>777</v>
       </c>
       <c r="E383" t="s">
         <v>776</v>
       </c>
-      <c r="J383" s="49"/>
-      <c r="K383" s="49"/>
     </row>
     <row r="384" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A384" t="s">
@@ -13807,7 +13528,7 @@
       <c r="C384" t="s">
         <v>1466</v>
       </c>
-      <c r="D384" s="43" t="s">
+      <c r="D384" s="15" t="s">
         <v>1467</v>
       </c>
       <c r="E384" t="s">
@@ -13824,7 +13545,7 @@
       <c r="C385" s="4" t="s">
         <v>1469</v>
       </c>
-      <c r="D385" s="43" t="s">
+      <c r="D385" s="15" t="s">
         <v>1467</v>
       </c>
       <c r="E385" t="s">
@@ -13844,7 +13565,7 @@
       <c r="C386" t="s">
         <v>1250</v>
       </c>
-      <c r="D386" s="43" t="s">
+      <c r="D386" s="15" t="s">
         <v>1251</v>
       </c>
       <c r="E386" t="s">
@@ -13861,7 +13582,7 @@
       <c r="C387" t="s">
         <v>625</v>
       </c>
-      <c r="D387" s="43" t="s">
+      <c r="D387" s="15" t="s">
         <v>626</v>
       </c>
       <c r="E387" t="s">
@@ -13878,7 +13599,7 @@
       <c r="C388" t="s">
         <v>562</v>
       </c>
-      <c r="D388" s="43" t="s">
+      <c r="D388" s="15" t="s">
         <v>563</v>
       </c>
       <c r="E388" t="s">
@@ -13895,122 +13616,149 @@
       <c r="C389" t="s">
         <v>423</v>
       </c>
-      <c r="D389" s="43" t="s">
+      <c r="D389" s="15" t="s">
         <v>424</v>
       </c>
       <c r="E389" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="390" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B390" s="17" t="s">
+    <row r="390" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A390" s="47" t="s">
+        <v>1568</v>
+      </c>
+      <c r="B390" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C390" t="s">
+      <c r="C390" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D390" s="43" t="s">
+      <c r="D390" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="E390" t="s">
+      <c r="E390" s="21" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="391" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B391" s="17" t="s">
+    <row r="391" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A391" s="47" t="s">
+        <v>1569</v>
+      </c>
+      <c r="B391" s="47" t="s">
         <v>840</v>
       </c>
-      <c r="C391" t="s">
+      <c r="C391" s="21" t="s">
         <v>841</v>
       </c>
-      <c r="D391" s="43" t="s">
+      <c r="D391" s="48" t="s">
         <v>842</v>
       </c>
-      <c r="E391" t="s">
+      <c r="E391" s="21" t="s">
         <v>841</v>
       </c>
     </row>
-    <row r="392" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B392" s="17" t="s">
+    <row r="392" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A392" s="47" t="s">
+        <v>1570</v>
+      </c>
+      <c r="B392" s="47" t="s">
         <v>337</v>
       </c>
-      <c r="C392" t="s">
+      <c r="C392" s="21" t="s">
         <v>338</v>
       </c>
-      <c r="D392" s="43" t="s">
+      <c r="D392" s="48" t="s">
         <v>339</v>
       </c>
-      <c r="E392" t="s">
+      <c r="E392" s="21" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="393" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B393" s="17" t="s">
+    <row r="393" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A393" s="47" t="s">
+        <v>1571</v>
+      </c>
+      <c r="B393" s="47" t="s">
         <v>203</v>
       </c>
-      <c r="C393" t="s">
+      <c r="C393" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="D393" s="43" t="s">
+      <c r="D393" s="48" t="s">
         <v>205</v>
       </c>
-      <c r="E393" t="s">
+      <c r="E393" s="21" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="394" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B394" s="17" t="s">
+    <row r="394" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A394" s="47" t="s">
+        <v>1572</v>
+      </c>
+      <c r="B394" s="47" t="s">
         <v>215</v>
       </c>
-      <c r="C394" t="s">
+      <c r="C394" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="D394" s="43" t="s">
+      <c r="D394" s="48" t="s">
         <v>217</v>
       </c>
-      <c r="E394" t="s">
+      <c r="E394" s="21" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="395" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B395" s="17" t="s">
+    <row r="395" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A395" s="47" t="s">
+        <v>1573</v>
+      </c>
+      <c r="B395" s="47" t="s">
         <v>1042</v>
       </c>
-      <c r="C395" t="s">
+      <c r="C395" s="21" t="s">
         <v>1043</v>
       </c>
-      <c r="D395" s="43" t="s">
+      <c r="D395" s="48" t="s">
         <v>1044</v>
       </c>
-      <c r="E395" t="s">
+      <c r="E395" s="21" t="s">
         <v>1043</v>
       </c>
-    </row>
-    <row r="396" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B396" t="s">
+      <c r="F395" s="21" t="s">
+        <v>1574</v>
+      </c>
+    </row>
+    <row r="396" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A396" s="47" t="s">
+        <v>1575</v>
+      </c>
+      <c r="B396" s="21" t="s">
         <v>519</v>
       </c>
-      <c r="C396" t="s">
+      <c r="C396" s="21" t="s">
         <v>520</v>
       </c>
-      <c r="D396" s="43" t="s">
+      <c r="D396" s="48" t="s">
         <v>521</v>
       </c>
-      <c r="E396" t="s">
+      <c r="E396" s="21" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="397" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B397" t="s">
+    <row r="397" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A397" s="47" t="s">
+        <v>1576</v>
+      </c>
+      <c r="B397" s="21" t="s">
         <v>692</v>
       </c>
-      <c r="C397" t="s">
+      <c r="C397" s="21" t="s">
         <v>693</v>
       </c>
-      <c r="D397" s="43" t="s">
+      <c r="D397" s="48" t="s">
         <v>694</v>
       </c>
-      <c r="E397" t="s">
+      <c r="E397" s="21" t="s">
         <v>693</v>
       </c>
     </row>
@@ -14024,7 +13772,7 @@
       <c r="C398" s="33" t="s">
         <v>440</v>
       </c>
-      <c r="D398" s="48" t="s">
+      <c r="D398" s="46" t="s">
         <v>441</v>
       </c>
       <c r="E398" s="33" t="s">
@@ -14042,7 +13790,7 @@
       <c r="C399" s="33" t="s">
         <v>865</v>
       </c>
-      <c r="D399" s="48" t="s">
+      <c r="D399" s="46" t="s">
         <v>866</v>
       </c>
       <c r="E399" s="33" t="s">
@@ -14060,7 +13808,7 @@
       <c r="C400" s="33" t="s">
         <v>869</v>
       </c>
-      <c r="D400" s="48" t="s">
+      <c r="D400" s="46" t="s">
         <v>870</v>
       </c>
       <c r="E400" s="33" t="s">
@@ -14078,7 +13826,7 @@
       <c r="C401" s="33" t="s">
         <v>873</v>
       </c>
-      <c r="D401" s="48" t="s">
+      <c r="D401" s="46" t="s">
         <v>874</v>
       </c>
       <c r="E401" s="33" t="s">
@@ -14096,7 +13844,7 @@
       <c r="C402" s="33" t="s">
         <v>915</v>
       </c>
-      <c r="D402" s="48" t="s">
+      <c r="D402" s="46" t="s">
         <v>916</v>
       </c>
       <c r="E402" s="33" t="s">
@@ -14114,7 +13862,7 @@
       <c r="C403" s="34" t="s">
         <v>861</v>
       </c>
-      <c r="D403" s="48" t="s">
+      <c r="D403" s="46" t="s">
         <v>862</v>
       </c>
       <c r="E403" s="34" t="s">
@@ -14132,7 +13880,7 @@
       <c r="C404" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="D404" s="48" t="s">
+      <c r="D404" s="46" t="s">
         <v>22</v>
       </c>
       <c r="E404" s="34" t="s">

</xml_diff>